<commit_message>
chore: cleanup temp files and organize scripts
- Delete LLM benchmark scripts (performance gain: none)
- Delete Gemini embedder test results (BGE > Gemini: 0.8693 vs 0.8466)
- Add scripts/README.md with categorized index (99 scripts in 10 categories)
- Clean test_results folder (keep only production outputs)
- Maintain PA optimal config: bt=0.639, bf=0.89, sp=0.00016
</commit_message>
<xml_diff>
--- a/archive/deprecated_2026_01_13/bsp_weight_grid_half_seed1_ex250/_preflight/bt0.70_pB0.400_pS0.400_sT0.000_sC0.000/seed1/pa_test_input_seed1.xlsx
+++ b/archive/deprecated_2026_01_13/bsp_weight_grid_half_seed1_ex250/_preflight/bt0.70_pB0.400_pS0.400_sT0.000_sC0.000/seed1/pa_test_input_seed1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D81"/>
+  <dimension ref="A1:D101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -772,36 +772,36 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>208</v>
+        <v>168</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>或以問臣軾호되 上與太皇太后 安所施設而及此오 臣軾對曰 在易大有上九에 自天祐之하야 吉無不利라한대 孔子曰 天之所助者는 順也요 人之所助者는 信也니 履信思乎順하고 又以尙賢也라 是以로 自天祐之하야 吉無不利라하시니라 今二聖이 躬信順以先天下하시고 而用司馬公하야 以致天下士하야 應是三德矣시니라 且以臣觀之컨대 公은 仁人也니 天相之矣시니라</t>
+          <t>及至秦, 漢之世하야는 其民이 見利而忘義하고 見危而不能授命이라 法禁之所不及이면 則巧僞變詐 無所不爲하고 疾視其長上하야 而幸其災하니 因之以水旱하고 加之以盜賊이면 則天下蕩然하야 無復天子之民矣니이다</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>혹자가 이것을 가지고 신(臣) 소식(蘇軾)에게 묻기를 “성상(聖上)과 태황태후께서 무슨 일을 시행하셨기에 여기에 이른 것입니까? ”라고 하기에, 신(臣) 소식(蘇軾)은 다음과 같이 대답하였다. “≪주역(周易)≫ 대유괘(大有卦) 상구(上九) 효사(爻辭)에 ‘하늘이 도와주어 길(吉)하여 이롭지 않음이 없다. ’라고 하였는데, 공자(孔子)께서 말씀하시기를 ‘하늘이 도와주는 것은 순함이요(천리(天理)에 순응하는 자이고) 사람이 도와주는 것은 성실함이니(성실한 자이니), 성실함을 이행하고 순함을 생각하고 또 어진 이를 높인다. 이 때문에 하늘이 도와주어 길(吉)하여 이롭지 않음이 없는 것이다. ’라고 하셨다. 그런데 지금 두 성상(聖上)께서 몸소 성실함과 순함으로 천하(天下)에 솔선하시고, 사마공(司馬公)을 등용하고 천하(天下)의 선비들을 초치하시어 이 세 가지 덕(德)에 응하신 것이다. 또 신(臣)의 입장에서 보건대, 공(公)은 인인(仁人)이시니 하늘이 도우시는 것이다. ”</t>
+          <t>그런데 진(秦)․한(漢) 시대(時代)에 이르러서는 백성들이 이익을 보면 의(義)를 잊고, 나라의 위태로움을 보고도 목숨을 바치지 않았습니다. 그래서 법과 금령이 미치지 않는 곳에는 공교롭게 거짓말하고 임기응변으로 속이는 짓을 하지 않는 바가 없고, 장상(長上)을 미워하고 원망하여 그에게 재앙이 일어나기를 바랐으니, 이로 인해 수해와 한해가 뒤따르고 겸하여 도적이 일어나면 천하(天下) 사람들이 다 없어져서 다시는 천자(天子)의 백성이 없게 되었습니다.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>당송팔대가문초소식5</t>
+          <t>당송팔대가문초소식4</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>369</v>
+        <v>208</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>昔我先子 沒於東京에 公爲二詩하야 以祖其行하니 文追典誥하고 論極皇王이라 公言一出에 孰敢改評이리오</t>
+          <t>或以問臣軾호되 上與太皇太后 安所施設而及此오 臣軾對曰 在易大有上九에 自天祐之하야 吉無不利라한대 孔子曰 天之所助者는 順也요 人之所助者는 信也니 履信思乎順하고 又以尙賢也라 是以로 自天祐之하야 吉無不利라하시니라 今二聖이 躬信順以先天下하시고 而用司馬公하야 以致天下士하야 應是三德矣시니라 且以臣觀之컨대 公은 仁人也니 天相之矣시니라</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>옛날 우리 선친(소순(蘇洵))께서 동경(東京)에서 별세하시자, 공(公)은 만시(挽詩) 두 수를 지어서 상여 길을 전송하시니, 문장은 전고(典誥)를 따르고 의논은 삼황(三皇)․오제(五帝)를 지극히 하셨습니다. 공(公)의 말씀이 한 번 나오니, 누가 감히 고치고 평하겠습니까?</t>
+          <t>혹자가 이것을 가지고 신(臣) 소식(蘇軾)에게 묻기를 “성상(聖上)과 태황태후께서 무슨 일을 시행하셨기에 여기에 이른 것입니까? ”라고 하기에, 신(臣) 소식(蘇軾)은 다음과 같이 대답하였다. “≪주역(周易)≫ 대유괘(大有卦) 상구(上九) 효사(爻辭)에 ‘하늘이 도와주어 길(吉)하여 이롭지 않음이 없다. ’라고 하였는데, 공자(孔子)께서 말씀하시기를 ‘하늘이 도와주는 것은 순함이요(천리(天理)에 순응하는 자이고) 사람이 도와주는 것은 성실함이니(성실한 자이니), 성실함을 이행하고 순함을 생각하고 또 어진 이를 높인다. 이 때문에 하늘이 도와주어 길(吉)하여 이롭지 않음이 없는 것이다. ’라고 하셨다. 그런데 지금 두 성상(聖上)께서 몸소 성실함과 순함으로 천하(天下)에 솔선하시고, 사마공(司馬公)을 등용하고 천하(天下)의 선비들을 초치하시어 이 세 가지 덕(德)에 응하신 것이다. 또 신(臣)의 입장에서 보건대, 공(公)은 인인(仁人)이시니 하늘이 도우시는 것이다. ”</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -812,16 +812,16 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>400</v>
+        <v>369</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>書黃子思詩集後 公之詩不入詩家品題로되 而其論詩處는 興味自遠하니라</t>
+          <t>昔我先子 沒於東京에 公爲二詩하야 以祖其行하니 文追典誥하고 論極皇王이라 公言一出에 孰敢改評이리오</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>황자사(黃子思)의 시집(詩集) 뒤에 쓰다 공(公)(東坡)의 시(詩)는 시가(詩家)의 품제(品題)에 들지 못하였으나, 시(詩)를 논한 곳은 흥미(興味)가 절로 원대하다.</t>
+          <t>옛날 우리 선친(소순(蘇洵))께서 동경(東京)에서 별세하시자, 공(公)은 만시(挽詩) 두 수를 지어서 상여 길을 전송하시니, 문장은 전고(典誥)를 따르고 의논은 삼황(三皇)․오제(五帝)를 지극히 하셨습니다. 공(公)의 말씀이 한 번 나오니, 누가 감히 고치고 평하겠습니까?</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -832,36 +832,36 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>93</v>
+        <v>400</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>蘇氏兄弟所見이 俱如此니라</t>
+          <t>書黃子思詩集後 公之詩不入詩家品題로되 而其論詩處는 興味自遠하니라</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>소씨형제(蘇氏兄弟)의 소견(所見)이 모두 이와 같았다.</t>
+          <t>황자사(黃子思)의 시집(詩集) 뒤에 쓰다 공(公)(東坡)의 시(詩)는 시가(詩家)의 품제(品題)에 들지 못하였으나, 시(詩)를 논한 곳은 흥미(興味)가 절로 원대하다.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>당송팔대가문초소철1</t>
+          <t>당송팔대가문초소식5</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>243</v>
+        <v>93</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>天下之事는 急之則喪하고 緩之則得이나 而過緩則無及이니이다 孔子曰 道之難行也를 我知之矣로니 知者는 過之하고 不肖者는 不及也일새니라하시니이다 夫天下患於不知요 而又有知而過之者하니 則是道之果難行也니이다 昔者엔 世之賢人이 患夫世之愛其爵祿하되 而不忍以其身으로 嘗試於艱難也니이다 故로 其上之人은 奮不顧身하고 以搏天下之公利而忘其私니이다 在下者도 亦不敢自愛하고 叫號紛呶하여 以攻訐其上之短이니이다 是二者는 可謂賢於天下之士矣로되 而猶未免爲不知니이다 何者오 不知自安其身之爲安天下之人이요 自重其發之爲重君子之勢하고 而輕用之於尋常之事니 則是猶匹夫之亮耳니이다</t>
+          <t>蘇氏兄弟所見이 俱如此니라</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>천하(天下)의 모든 일은 급하면 상실하게 되고 느슨하면 얻게 되나, 지나치게 느슨하면 한 가지 일도 이루지 못합니다. 공자(孔子)가 말하기를 “도(道)가 행해지기 어려운 이유를 내가 아노니, 아는 사람은 지나치고 어질지 못한 사람은 미치지 못하기 때문이다. ”라고 하였습니다. 대체로 천하(天下) 사람들은 알지 못하는 것을 병폐로 여기고, 또 알면서 지나친 자가 있으니, 이래서 도(道)가 종시 행하기 어려운 것입니다. 옛날에는 세상의 현인(賢人)이 세상에서 작록(爵祿)을 애호하되 차마 자기 몸으로 간난(艱難)을 겪지 않는 것을 병폐로 여겼습니다. 그러므로 위에 있는 사람은 분연(奮然)히 일어나 자신을 고석(顧惜)하지 않은 채 천하의 공리(公利)를 취하고 자신의 이익은 잊었습니다. 아래에 있는 사람도 감히 자신을 아끼지 않은 채 큰소리치며 윗사람의 단점을 들추었습니다. 이 두 사람은 천하의 선비보다 낫다고 할 수 있겠으나 오히려 알지 못한 것을 면치 못하였습니다. 왜냐하면, 자신을 편안하게 하는 것이 바로 천하 사람을 편안하게 하는 것이고, 자신의 행동을 자중하는 것이 바로 군자의 처신을 신중하게 하는 것임을 알지 못하고 가벼이 사소한 일에 신경을 썼으니, 이는 무식한 사람이나 인정할 일입니다.</t>
+          <t>소씨형제(蘇氏兄弟)의 소견(所見)이 모두 이와 같았다.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -872,16 +872,16 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>291</v>
+        <v>243</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>然이나 劉項은 奮臂於閭閻之中하여 率天下蜂起之兵하고 西嚮以攻秦이니라 無一成之聚와 一夫之衆하고 驅罷敝謫戍之人하여 以求所非望하니 得之則生이요 失之則死라 以匹夫而圖天下는 其勢不得不疾戰以趨利니라 是以로 冒萬死求一生而不顧니라 今秦은 擁千里之地하고 而乘累世之業이니 雖閉關而守之하여 畜威養兵하고 拊循士卒이라도 而諸侯誰敢謀秦이리오 觀天下之釁而後에 出兵以乘其弊라도 天下夫誰敢抗이리오마는 而惠文武昭之君은 乃以萬乘之資로 而用匹夫所以圖天下之勢하여 疾戰而不顧其後하니 此宜其能以取天下나 而亦能以亡之也니라</t>
+          <t>天下之事는 急之則喪하고 緩之則得이나 而過緩則無及이니이다 孔子曰 道之難行也를 我知之矣로니 知者는 過之하고 不肖者는 不及也일새니라하시니이다 夫天下患於不知요 而又有知而過之者하니 則是道之果難行也니이다 昔者엔 世之賢人이 患夫世之愛其爵祿하되 而不忍以其身으로 嘗試於艱難也니이다 故로 其上之人은 奮不顧身하고 以搏天下之公利而忘其私니이다 在下者도 亦不敢自愛하고 叫號紛呶하여 以攻訐其上之短이니이다 是二者는 可謂賢於天下之士矣로되 而猶未免爲不知니이다 何者오 不知自安其身之爲安天下之人이요 自重其發之爲重君子之勢하고 而輕用之於尋常之事니 則是猶匹夫之亮耳니이다</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>그러나 유방(劉邦)과 항적(項籍)은 여염(閭閻)(민간(民間))에서 팔을 걷어붙이고 대사(大事)를 일으켜 천하(天下)에서 봉기(蜂起)한 군사들을 거느리고 서쪽을 향하여 진(秦)을 공격하였다. 조그마한 촌락(村落)이나 한 명의 인민도 확보한 지반(地盤)이 없는 상태에서 적벌(謫罰)로 괴롭게 변방에서 수자리하는 사람들을 몰아서 분수 밖의 소원을 구하였으니, 천하(天下)를 얻으면 생존하고 전투에서 패전하면 사망하기 마련이므로 필부(匹夫)로서 천하(天下)를 도모하는 것은 그 형세에 있어서 부득불 빨리 서둘러 싸워서 생존하기를 구해야만 했다. 그렇기 때문에 만 번 죽음을 무릅쓰고 한 번 생존하기를 구하여 다른 것을 돌아볼 겨를이 없었다. 당시 진(秦)은 천리나 되는 땅을 점유하고, 여러 세대의 공업(功業)을 빙자하였으니, 비록 함곡관(函谷關)만 지키며 군사의 위용과 사기를 기르고 사졸(士卒)(군민(軍民))들을 편하게 어루만진다 하더라도 제후(諸侯) 중에 그 누가 감히 진(秦)을 도모하겠는가? 천하(天下)에 전란이 발생하는 것을 관망하고 나서 서서히 군사를 출동하여 제후(諸侯)들이 피곤에 지친 틈을 타 공격한다 하더라도 천하에 누가 감히 저항하겠는가? 그런데 혜문왕(惠文王)‧도무왕(悼武王)‧소왕(昭王) 같은 군주(君主)는 제왕(帝王)의 자격으로 필부(匹夫)가 천하(天下)를 도모하기 위하여 뒤도 돌아보지 않은 채 빨리 서둘러 전쟁을 하는 방법을 취하였으니, 이 방법은 천하(天下)를 취득할 수도 있지만 또한 망하게 할 수도 있는 것이다.</t>
+          <t>천하(天下)의 모든 일은 급하면 상실하게 되고 느슨하면 얻게 되나, 지나치게 느슨하면 한 가지 일도 이루지 못합니다. 공자(孔子)가 말하기를 “도(道)가 행해지기 어려운 이유를 내가 아노니, 아는 사람은 지나치고 어질지 못한 사람은 미치지 못하기 때문이다. ”라고 하였습니다. 대체로 천하(天下) 사람들은 알지 못하는 것을 병폐로 여기고, 또 알면서 지나친 자가 있으니, 이래서 도(道)가 종시 행하기 어려운 것입니다. 옛날에는 세상의 현인(賢人)이 세상에서 작록(爵祿)을 애호하되 차마 자기 몸으로 간난(艱難)을 겪지 않는 것을 병폐로 여겼습니다. 그러므로 위에 있는 사람은 분연(奮然)히 일어나 자신을 고석(顧惜)하지 않은 채 천하의 공리(公利)를 취하고 자신의 이익은 잊었습니다. 아래에 있는 사람도 감히 자신을 아끼지 않은 채 큰소리치며 윗사람의 단점을 들추었습니다. 이 두 사람은 천하의 선비보다 낫다고 할 수 있겠으나 오히려 알지 못한 것을 면치 못하였습니다. 왜냐하면, 자신을 편안하게 하는 것이 바로 천하 사람을 편안하게 하는 것이고, 자신의 행동을 자중하는 것이 바로 군자의 처신을 신중하게 하는 것임을 알지 못하고 가벼이 사소한 일에 신경을 썼으니, 이는 무식한 사람이나 인정할 일입니다.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -892,96 +892,96 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>12</v>
+        <v>291</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>今夫隋文之世에도 其亦見天下之久不定하고 而重失其定也니라 蓋自東晉以來로 劉聰石勒慕容垂苻堅姚興赫連之徒 紛紛而起者 不可勝數니라 至於元氏하여는 幷呑滅取하여 略已盡矣나 而南方未服이니라 元氏自分而爲周齊하고 周幷齊而授之隋하고 隋文取梁滅陳하니 而後에 天下爲一이니라 彼亦見天下之久不定也라 是以로 旣得天下之衆이나 而恐其失之하고 享天下之樂이나 而懼其不久하고 立於萬民之上이나 而常有猜防不安之心하여 以爲擧世之人이 皆有曩者英雄割據之懷라하고 制爲嚴法峻令하여 以杜天下之變하며 謀臣舊將을 誅滅略盡하고 而獨死於楊素之手하여 以及於大故하며 終於煬帝之際에 天下大亂하여 塗地而莫之救니라 由此觀之면 則夫隋之所以亡者는 無以異於秦也니라</t>
+          <t>然이나 劉項은 奮臂於閭閻之中하여 率天下蜂起之兵하고 西嚮以攻秦이니라 無一成之聚와 一夫之衆하고 驅罷敝謫戍之人하여 以求所非望하니 得之則生이요 失之則死라 以匹夫而圖天下는 其勢不得不疾戰以趨利니라 是以로 冒萬死求一生而不顧니라 今秦은 擁千里之地하고 而乘累世之業이니 雖閉關而守之하여 畜威養兵하고 拊循士卒이라도 而諸侯誰敢謀秦이리오 觀天下之釁而後에 出兵以乘其弊라도 天下夫誰敢抗이리오마는 而惠文武昭之君은 乃以萬乘之資로 而用匹夫所以圖天下之勢하여 疾戰而不顧其後하니 此宜其能以取天下나 而亦能以亡之也니라</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>지금 수(隋) 문제(文帝)의 세대 또한 천하(天下)가 오래 안정되지 못함을 보고서도 거듭 그 안정을 잃었다. 대개 동진(東晉) 이래로 유총(劉聰), 석륵(石勒), 모용수(慕容垂), 부견(苻堅), 요흥(姚興), 혁련(赫連)과 같은 무리가 어지럽게 일어난 경우는 이루 다 셀 수가 없다. 원씨(元氏)에 이르러서 병탄(幷呑)하고 멸취(滅取)하여 천하를 이미 다 보유하였지만, 남쪽 지방은 복종시키지 못하였다. 원씨(元氏)는 스스로 나뉘어 주(周)나라와 제(齊)나라가 되었고, 주(周)나라는 제(齊)나라를 아울러 수(隋)나라에 넘겨주었고, 수(隋) 문제(文帝)는 양(梁)나라를 취하고 진(陳)나라를 멸하였으니, 그렇게 한 뒤에야 천하(天下)가 통일될 수 있었다. 수(隋) 문제(文帝) 또한 천하(天下)가 오래 안정되지 못함을 보았다. 그래서 이미 천하(天下)의 민중을 얻었으나 그것을 잃을까 두려워하였고, 천하(天下)의 낙(樂)을 누렸으나 그것이 오래가지 못할까 두려워하였고, 만백성의 위에 군림하였으나 항상 의심하고 대비하느라 불안한 마음을 가져, 온 세상 사람들이 모두 이전 영웅들처럼 할거(割據)할 생각을 품는다고 여기고 준엄한 법령을 제정하여 천하(天下)의 변(變)을 막았으며, 모신(謀臣)과 구장(舊將)을 주멸(誅滅)하여 모두 없애고, 자신은 양소(楊素)의 손에서 죽어 큰 화환(禍患)이 이르게 하였으며, 끝내는 양제(煬帝) 때에 천하(天下)가 크게 혼란하여 여지없이 파괴되었는데도 구제하지 못하였다. 이것을 가지고 본다면 수(隋)나라가 망한 까닭도 진(秦)나라와 다를 것이 없었다.</t>
+          <t>그러나 유방(劉邦)과 항적(項籍)은 여염(閭閻)(민간(民間))에서 팔을 걷어붙이고 대사(大事)를 일으켜 천하(天下)에서 봉기(蜂起)한 군사들을 거느리고 서쪽을 향하여 진(秦)을 공격하였다. 조그마한 촌락(村落)이나 한 명의 인민도 확보한 지반(地盤)이 없는 상태에서 적벌(謫罰)로 괴롭게 변방에서 수자리하는 사람들을 몰아서 분수 밖의 소원을 구하였으니, 천하(天下)를 얻으면 생존하고 전투에서 패전하면 사망하기 마련이므로 필부(匹夫)로서 천하(天下)를 도모하는 것은 그 형세에 있어서 부득불 빨리 서둘러 싸워서 생존하기를 구해야만 했다. 그렇기 때문에 만 번 죽음을 무릅쓰고 한 번 생존하기를 구하여 다른 것을 돌아볼 겨를이 없었다. 당시 진(秦)은 천리나 되는 땅을 점유하고, 여러 세대의 공업(功業)을 빙자하였으니, 비록 함곡관(函谷關)만 지키며 군사의 위용과 사기를 기르고 사졸(士卒)(군민(軍民))들을 편하게 어루만진다 하더라도 제후(諸侯) 중에 그 누가 감히 진(秦)을 도모하겠는가? 천하(天下)에 전란이 발생하는 것을 관망하고 나서 서서히 군사를 출동하여 제후(諸侯)들이 피곤에 지친 틈을 타 공격한다 하더라도 천하에 누가 감히 저항하겠는가? 그런데 혜문왕(惠文王)‧도무왕(悼武王)‧소왕(昭王) 같은 군주(君主)는 제왕(帝王)의 자격으로 필부(匹夫)가 천하(天下)를 도모하기 위하여 뒤도 돌아보지 않은 채 빨리 서둘러 전쟁을 하는 방법을 취하였으니, 이 방법은 천하(天下)를 취득할 수도 있지만 또한 망하게 할 수도 있는 것이다.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>당송팔대가문초소철2</t>
+          <t>당송팔대가문초소철1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>158</v>
+        <v>12</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>平糴屯田이니라 今策士도 亦當擧其說하여 以獻於天子니라</t>
+          <t>今夫隋文之世에도 其亦見天下之久不定하고 而重失其定也니라 蓋自東晉以來로 劉聰石勒慕容垂苻堅姚興赫連之徒 紛紛而起者 不可勝數니라 至於元氏하여는 幷呑滅取하여 略已盡矣나 而南方未服이니라 元氏自分而爲周齊하고 周幷齊而授之隋하고 隋文取梁滅陳하니 而後에 天下爲一이니라 彼亦見天下之久不定也라 是以로 旣得天下之衆이나 而恐其失之하고 享天下之樂이나 而懼其不久하고 立於萬民之上이나 而常有猜防不安之心하여 以爲擧世之人이 皆有曩者英雄割據之懷라하고 制爲嚴法峻令하여 以杜天下之變하며 謀臣舊將을 誅滅略盡하고 而獨死於楊素之手하여 以及於大故하며 終於煬帝之際에 天下大亂하여 塗地而莫之救니라 由此觀之면 則夫隋之所以亡者는 無以異於秦也니라</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>평적(平糴)과 둔전(屯田)에 대한 논술이다. 오늘날의 책사(策士)도 마땅히 그 설(說)을 들어서 천자(天子)에게 드려야 하겠다.</t>
+          <t>지금 수(隋) 문제(文帝)의 세대 또한 천하(天下)가 오래 안정되지 못함을 보고서도 거듭 그 안정을 잃었다. 대개 동진(東晉) 이래로 유총(劉聰), 석륵(石勒), 모용수(慕容垂), 부견(苻堅), 요흥(姚興), 혁련(赫連)과 같은 무리가 어지럽게 일어난 경우는 이루 다 셀 수가 없다. 원씨(元氏)에 이르러서 병탄(幷呑)하고 멸취(滅取)하여 천하를 이미 다 보유하였지만, 남쪽 지방은 복종시키지 못하였다. 원씨(元氏)는 스스로 나뉘어 주(周)나라와 제(齊)나라가 되었고, 주(周)나라는 제(齊)나라를 아울러 수(隋)나라에 넘겨주었고, 수(隋) 문제(文帝)는 양(梁)나라를 취하고 진(陳)나라를 멸하였으니, 그렇게 한 뒤에야 천하(天下)가 통일될 수 있었다. 수(隋) 문제(文帝) 또한 천하(天下)가 오래 안정되지 못함을 보았다. 그래서 이미 천하(天下)의 민중을 얻었으나 그것을 잃을까 두려워하였고, 천하(天下)의 낙(樂)을 누렸으나 그것이 오래가지 못할까 두려워하였고, 만백성의 위에 군림하였으나 항상 의심하고 대비하느라 불안한 마음을 가져, 온 세상 사람들이 모두 이전 영웅들처럼 할거(割據)할 생각을 품는다고 여기고 준엄한 법령을 제정하여 천하(天下)의 변(變)을 막았으며, 모신(謀臣)과 구장(舊將)을 주멸(誅滅)하여 모두 없애고, 자신은 양소(楊素)의 손에서 죽어 큰 화환(禍患)이 이르게 하였으며, 끝내는 양제(煬帝) 때에 천하(天下)가 크게 혼란하여 여지없이 파괴되었는데도 구제하지 못하였다. 이것을 가지고 본다면 수(隋)나라가 망한 까닭도 진(秦)나라와 다를 것이 없었다.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>당송팔대가문초소철3</t>
+          <t>당송팔대가문초소철2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>中使宣醫謝表</t>
+          <t>平糴屯田이니라 今策士도 亦當擧其說하여 以獻於天子니라</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>환관을 보내어 선지(宣旨)로 어의(御醫)를 파견하신데 감사하는 표(表)</t>
+          <t>평적(平糴)과 둔전(屯田)에 대한 논술이다. 오늘날의 책사(策士)도 마땅히 그 설(說)을 들어서 천자(天子)에게 드려야 하겠다.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>당송팔대가문초왕안석1</t>
+          <t>당송팔대가문초소철3</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>116</v>
+        <v>153</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>或問復讐어늘 對曰 非治世之道也라 明天子在上하고 自方伯諸侯로 以至於有司히 各修其職이면 其能殺不辜者少矣니라 不幸而有焉이면 則其子弟以告于有司하고 有司不能聽이면 以告于其君하고 其君不能聽이면 以告于方伯하고 方伯不能聽이면 以告于天子하나니 則天子誅其不能聽者하고 而爲之施刑於其讐하나니라 亂世則天子諸侯方伯에 皆不可以告라 故書說紂曰 凡有辜罪 乃罔恒獲한대 小民方興하야 相爲敵讐라하니 蓋讐之所以興이어늘 以上之不可告하고 辜罪之不常獲也니라 方是時하야 有父兄之讐하야 而輒殺之者면 君子權其勢하야 恕其情而與之可也라 故復讐之義 見於春秋傳하고 見於禮記하니 爲亂世之爲子弟者言之也니라</t>
+          <t>中使宣醫謝表</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>어떤 사람이 원수를 갚는 일에 대하여 묻기에, 대답하기를 “잘 다스려지는 시대에 썼던 방도가 아니다. ”라고 하였다. 밝으신 천자(天子)께서 위에 계시고, 방백(方伯)과 제후(諸侯)로부터 담당관서에 이르기까지 각기 그들이 맡은 직무를 잘 처리하면, 허물이 없는 사람을 죽이는 경우가 드물게 된다. 불행하게도 그런 경우가 있으면, 그 자제들이 이를 담당관서에 알리고, 담당관서에서 들어주지 않으면 이를 제후에게 알리고, 제후가 들어주지 않으면 이를 방백에게 알리고, 방백이 들어주지 않으면 이를 천자께 고한다. 그렇게 되면 천자는 들어주지 않았던 자를 징계하고, 그를 위하여 그 원수에게 형벌을 시행한다. 정치가 어지러운 시대에는 천자나 제후나 방백 등 누구에게도 이를 알릴 수가 없게 된다. 그러므로 《서경(書經)》에서 주(紂)에 대하여 말하기를 “무릇 죄악을 범한 자를 항상 잡아들이는 일이 없자, 소인배들이 사방에서 일어나 서로 대적하여 원수가 되었다. ” 하였으니, 이는 해치는 자들이 발흥하는데도 이를 위에 아뢸 수가 없고, 죄악을 범한 사람이 항시 잡히는 것도 아니었다. 바야흐로 그러한 때에는 부형(父兄)을 죽인 원수를 바로 보복하여 죽인 사람이 있으면, 통치자가 그 형세를 형량(衡量)해보아, 그 실정(實情)을 용인(容認)하고 이를 허여하는 것이 옳다. 그러므로 원수를 갚는 의의(意義)에 대한 것이 《춘추전(春秋傳)》에도 보이고, 《예기(禮記)》에도 보이는데, 이는 난세(亂世)에 부형(父兄)을 잃은 자제(子弟)를 위하여 말한 것이다.</t>
+          <t>환관을 보내어 선지(宣旨)로 어의(御醫)를 파견하신데 감사하는 표(表)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>당송팔대가문초왕안석2</t>
+          <t>당송팔대가문초왕안석1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>285</v>
+        <v>1</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>公李氏요 諱餘慶이며 字昌宗이니 年四十四에 官止國子博士 知常州以卒하다 然公之威名氣略은 聞天下하야 自其卒至今久矣로되 天下尙多談公之爲有過於人者하니라 余嘗過常州하니 州之長老道 公卒時就葬於橫山할새 州人塡道하야 瞻送歎息하고 爲之出淚하며 又爲之畫像하야 寘之浮屠以祭之하다 於是에 又知公之有惠愛於常人也호라 已而與公之子處厚遊하여 則得公之所爲甚具하다 蓋公之爲政에 精明强果하야 事至能立斷而得하야 久姦宿惡을 輒取之不貸하고 至其化服이면 則撫循養息하야 悉有其處라 所以威震遠近하야 而蒙其德者는 亦思之無窮也러라 當明肅太后時하야 嘗欲用公矣러니 公再上書論事하야 其言甚直하니 以故不果用 而出常州하다</t>
+          <t>周公論</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>공(公)은 이씨(李氏)로 휘(諱)는 여경(餘慶)이고 자(字)는 창종(昌宗)이며, 벼슬이 국자박사(國子博士) 지상주(知常州)에 이르렀던 44세에 졸(卒)하였다. 그러나 공(公)의 위명(威名)과 기략(氣略)은 천하에 소문이 나서, 졸(卒)한 이후 지금까지 오랜 기간이 지났지만, 천하에는 아직도 공(公)의 업적이 남보다 뛰어났던 점에 대하여 이야기하는 사람이 많이 있다. 내가 일찍이 상주(常州) 땅을 지날 때에 그 고을의 장로(長老)가 “공(公)이 졸(卒)하자 그때에 곧 횡산(橫山)에 안장(安葬)하였는데, 고을 사람들이 길이 메워지도록 모두 나와서 우러러 전송하며 탄식하고 그분을 위해 눈물을 흘렸고, 또 그분을 위해 초상화를 그려서 사원(寺院)에 안치하고 제사를 지내고 있다. ”라고 말하였으므로, 이에 공(公)이 상주(常州) 사람들에게 은혜를 입히고 사랑을 베풀었음을 더욱 잘 알게 되었다. 그 후 공(公)의 아드님 처후(處厚)와 교유하게 되어 공(公)이 한 일을 매우 자세히 알게 되었다. 대체로 공(公)이 정사(政事)를 베풀 때에 정밀하고 분명하며 꿋꿋하고 과단성이 있어서, 일의 처리에 이르러서는 단안(斷案)을 내려서 적의(適宜)함을 얻었고, 오랫동안 간사(奸邪)한 짓을 하거나 악독한 짓을 한 사람은 곧 잡아들여 용서 없이 벌을 주었으며, 백성들이 감화하여 순복함에 이르러서는 그들의 뜻에 맞게 안무(按撫)하고 길러주어, 모두가 안주(安住)할 곳이 있게 하였다. 이에 원근(遠近)에 위엄이 크게 떨치게 되었고, 그의 은덕을 입은 사람들이 또한 그를 무궁토록 그리워하게 되었다. 명숙태후(明肅太后)께서 수렴청정(垂簾聽政)할 때를 당하여, 일찍이 공(公)을 등용하고자 한 일이 있었는데, 공(公)이 거듭 상서(上書)하여 당시(當時)의 국사(國事)를 논하면서 그 말에 직언(直言)을 한 것이 매우 많았으므로, 이 때문에 공(公)의 임용이 실현되지 못하고 상주지사(常州知事)로 나가게 되었던 것이다.</t>
+          <t>주공에 대한 논</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -992,141 +992,141 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>富室은 貧之母也니 誠不可破壞라 然使其大倖而役於下는 則又不可니라 兄云懼富人流爲工商浮窳라하니 蓋甚急而不均이면 則有此耳라 若富者雖益賦라도 而其實輸當其十一이면 猶足安其堵하여 雖驅之不肯易也리라 檢之逾精이면 則下逾巧는 誠如兄之言이라 管子亦不欲以民産爲征이라 故有殺畜伐木之說하니라 今若非市井之征이면 則捨其産 而唯丁田之問이니 推以誠質하고 示以恩惠하며 嚴責吏以法이니라 如所陳一社一村之制를 遞以信相考면 安有不得其實이리오 不得其實이면 則一社一村之制도 亦不可行矣리라 是故乘弊政 必須一定制니 而後兄之說乃得行焉이니라 蒙之所見及此而已라 永州以僻隅로 少知人事라 兄之所代者는 誰耶아 理歟弊歟아 理則其說行矣어니와 若其弊也면 蒙之說其在可用之數乎인저</t>
+          <t>或問復讐어늘 對曰 非治世之道也라 明天子在上하고 自方伯諸侯로 以至於有司히 各修其職이면 其能殺不辜者少矣니라 不幸而有焉이면 則其子弟以告于有司하고 有司不能聽이면 以告于其君하고 其君不能聽이면 以告于方伯하고 方伯不能聽이면 以告于天子하나니 則天子誅其不能聽者하고 而爲之施刑於其讐하나니라 亂世則天子諸侯方伯에 皆不可以告라 故書說紂曰 凡有辜罪 乃罔恒獲한대 小民方興하야 相爲敵讐라하니 蓋讐之所以興이어늘 以上之不可告하고 辜罪之不常獲也니라 方是時하야 有父兄之讐하야 而輒殺之者면 君子權其勢하야 恕其情而與之可也라 故復讐之義 見於春秋傳하고 見於禮記하니 爲亂世之爲子弟者言之也니라</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>부유한 가구(家口)는 가난한 가구의 어머니이므로 파괴해선 안 됩니다. 그러나 그들로 하여금 너무 큰 요행을 얻게 하여 아랫사람들을 부리게 하는 것 또한 안 됩니다. 형은 부유한 사람이 공상업(工商業)으로 직업을 바꾸어 빈둥거리며 지낼까 두렵다고 하셨는데, 부자들에 대한 세금징수를 매우 급하게 하거나 공정하게 하지 않으면 이런 문제가 있을 것입니다. 만약 부자에게 비록 부세(賦稅)가 늘어나더라도 정말 소득의 10분의 1만 내도록 한다면 오히려 충분히 그 속에서 안주하고 〈공상업(工商業)으로〉 내몰더라도 본업(本業)을 바꾸려 하지 않을 것입니다. 관청에서 점검을 정밀하게 하면 할수록 아래의 부자가 세금을 도피하는 수법이 더욱 교묘해진다는 것은 참으로 형의 말씀이 맞습니다. 관자(管子) 역시 백성의 재산에 따라 징세하려고 하지 않았으므로 “가축을 죽이거나 나무를 베지 말게 하라. ”는 설이 있습니다. 지금 만약 시정(市井)의 상인(商人)에게 징세하지 않는다면 〈농가(農家)에 대해서도〉 그 재산에 따라 징세하는 것을 그만두고 오직 인구(人口)와 전답(田畓)을 따져 징세하여야 할 것이니, 백성을 성심(誠心)으로 대하고 〈이 방법이〉 혜택이 크다는 점을 알리는 한편 법률로 관리를 엄격하게 단속해야 합니다. 그러면서 형께서 말씀하신 것처럼 1사(社), 1촌(村)의 단위별로 실사(實査)하는 제도를 만들어 차례대로 확실하게 실사한다면, 어찌 실상을 파악하지 못하겠습니까. 실상을 파악하지 못한다면 1사(社), 1촌(村)의 제도 역시 시행할 수 없습니다. 그러므로 전임 수령의 부패한 정사를 이어받았을 경우에는 반드시 일정한 제도가 있어야 하니, 그래야만 형께서 말씀하신 방법이 시행될 수 있습니다. 저의 소견은 여기까지입니다. 영주(永州)는 구석진 곳이어서 바깥세상의 정황을 잘 모릅니다. 형의 전임자는 누구입니까? 잘 다스렸습니까, 부패하였습니까? 잘 다스렸다면 형께서 주장하신 설이 시행될 것이지만, 만약 부패하였다면 저의 건의가 어쩌면 채용될 수도 있을 것입니다.</t>
+          <t>어떤 사람이 원수를 갚는 일에 대하여 묻기에, 대답하기를 “잘 다스려지는 시대에 썼던 방도가 아니다. ”라고 하였다. 밝으신 천자(天子)께서 위에 계시고, 방백(方伯)과 제후(諸侯)로부터 담당관서에 이르기까지 각기 그들이 맡은 직무를 잘 처리하면, 허물이 없는 사람을 죽이는 경우가 드물게 된다. 불행하게도 그런 경우가 있으면, 그 자제들이 이를 담당관서에 알리고, 담당관서에서 들어주지 않으면 이를 제후에게 알리고, 제후가 들어주지 않으면 이를 방백에게 알리고, 방백이 들어주지 않으면 이를 천자께 고한다. 그렇게 되면 천자는 들어주지 않았던 자를 징계하고, 그를 위하여 그 원수에게 형벌을 시행한다. 정치가 어지러운 시대에는 천자나 제후나 방백 등 누구에게도 이를 알릴 수가 없게 된다. 그러므로 《서경(書經)》에서 주(紂)에 대하여 말하기를 “무릇 죄악을 범한 자를 항상 잡아들이는 일이 없자, 소인배들이 사방에서 일어나 서로 대적하여 원수가 되었다. ” 하였으니, 이는 해치는 자들이 발흥하는데도 이를 위에 아뢸 수가 없고, 죄악을 범한 사람이 항시 잡히는 것도 아니었다. 바야흐로 그러한 때에는 부형(父兄)을 죽인 원수를 바로 보복하여 죽인 사람이 있으면, 통치자가 그 형세를 형량(衡量)해보아, 그 실정(實情)을 용인(容認)하고 이를 허여하는 것이 옳다. 그러므로 원수를 갚는 의의(意義)에 대한 것이 《춘추전(春秋傳)》에도 보이고, 《예기(禮記)》에도 보이는데, 이는 난세(亂世)에 부형(父兄)을 잃은 자제(子弟)를 위하여 말한 것이다.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>당송팔대가문초유종원1</t>
+          <t>당송팔대가문초왕안석2</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>守令之於民에 近且重을 易知矣라 予嘗論今之守令컨대 有道而聞四方者는 不過數人이니 此數人者는 非特任守令也라 過此數人하여는 有千里者相接이로되 而無一賢守요 有百里者相環이로되 而無一賢令이라 至天子大臣이 嘗患其然하여는 則任奉法之吏하고 嚴刺察之科하여 以繩治之에 諸郡守縣令이 以罪不任職하여 或黜或罷者 相繼於外라 於是에 下詔書하여 擇廷臣하여 使各擧所知以任守令하니 是天子大臣愛國與民而重守令之意 可謂無不至矣라 而詔雖下나 擧者卒不聞하고 惟令或以舊制擧로 不偕循歲月而授라 每擧者有姓名을 得而視之하고 推考其材行能堪其擧者에 卒亦未見焉이라 擧者旣然矣니 則以余之所見聞으로 陰計其人之孰可擧者에 卒亦未見焉이라 猶恐余之愚且賤이 聞與見焉者少하여 不足以知天下之材也하여는 則求夫賢而有名位聞與見之博者하여 而從之問其人之孰可擧者에 卒亦未見焉이나 豈天下之人固可誣하고 而天固不生材於今哉아</t>
+          <t>公李氏요 諱餘慶이며 字昌宗이니 年四十四에 官止國子博士 知常州以卒하다 然公之威名氣略은 聞天下하야 自其卒至今久矣로되 天下尙多談公之爲有過於人者하니라 余嘗過常州하니 州之長老道 公卒時就葬於橫山할새 州人塡道하야 瞻送歎息하고 爲之出淚하며 又爲之畫像하야 寘之浮屠以祭之하다 於是에 又知公之有惠愛於常人也호라 已而與公之子處厚遊하여 則得公之所爲甚具하다 蓋公之爲政에 精明强果하야 事至能立斷而得하야 久姦宿惡을 輒取之不貸하고 至其化服이면 則撫循養息하야 悉有其處라 所以威震遠近하야 而蒙其德者는 亦思之無窮也러라 當明肅太后時하야 嘗欲用公矣러니 公再上書論事하야 其言甚直하니 以故不果用 而出常州하다</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>수령(守令)이 백성들에게 있어 가깝고도 중요하다는 사실은 알기 쉽다. 나는 오늘날의 수령들에 관해 일찍이 논해보았다. 이들 가운데 도덕이 몸에 배어 사방에 명성이 알려진 사람은 몇 사람에 지나지 않으니, 이 몇 사람은 그 능력이 수령직을 맡을 자격을 넘어선다. 이 몇 사람 외에 천 리 되는 지역을 맡은 자가 여기저기 깔려 있지만 누구 하나 어진 군수가 없으며, 백 리 되는 지역을 맡은 자가 꼬리를 물고 이어져 있지만 누구 하나 어진 현령이 없다. 천자와 대신들은 일찍이 이러한 현실에 대해 우려했다. 그리하여 법을 신봉하는 관리들을 임용하고 규찰하는 법을 엄격하게 적용하여 법률의 잣대로 그들을 치죄하자, 여러 군수와 현령들 가운데 죄 때문에 관직을 맡지 못하고 폐출되거나 파면된 이들이 지방에서 잇따라 나타나게 되었다. 이에 조서(詔書)를 내려 조정 대신을 골라 이들이 각자 자신이 알던 사람들을 천거하도록 하여 수령직을 맡게 했다. 이로 볼 때 천자와 대신들이 나라를 사랑하고 백성들과 함께하며 수령을 중시하는 뜻이 모두 다 지극하다 할 수 있을 것이다. 그러나 비록 조서(詔書)가 내려졌는데도 천거된 자가 있다는 말은 끝내 들리지 않았고, 오로지 현령만 간혹 기존의 제거(制擧)제도를 적용하고 재직한 연한과 이력에 따라 관직을 제수하지는 않는다. 매번 천거 대상자의 성명이 밝혀지면 그것을 보고 그의 재능과 행실이 천거를 받기에 충분한지를 따져보면 그런 자를 끝내 볼 수가 없다. 천거 대상자가 이미 그런 실정이기에 내가 보고 들을 사실을 근거로 그 사람들 중에 누가 천거할 만한 사람인지 속으로 헤아려보면 또한 끝내 그런 자를 볼 수가 없다. 우매하고 미천한 내가 문견이 적어 천하의 인재들을 충분히 알아보지 못할까 염려되기에,  현명하여 명망과 지위가 있고 문견의 범위가 넓은 자를 찾아가 지금 세상에 천거할 만한 자가 과연 누구이겠느냐고 물어보아도 끝내 그런 자를 볼 수가 없다. 그러나 어찌 천하 사람들을 무시할 수 있겠으며, 하늘이 과연 지금 세상에 인재를 내지 않았겠는가.</t>
+          <t>공(公)은 이씨(李氏)로 휘(諱)는 여경(餘慶)이고 자(字)는 창종(昌宗)이며, 벼슬이 국자박사(國子博士) 지상주(知常州)에 이르렀던 44세에 졸(卒)하였다. 그러나 공(公)의 위명(威名)과 기략(氣略)은 천하에 소문이 나서, 졸(卒)한 이후 지금까지 오랜 기간이 지났지만, 천하에는 아직도 공(公)의 업적이 남보다 뛰어났던 점에 대하여 이야기하는 사람이 많이 있다. 내가 일찍이 상주(常州) 땅을 지날 때에 그 고을의 장로(長老)가 “공(公)이 졸(卒)하자 그때에 곧 횡산(橫山)에 안장(安葬)하였는데, 고을 사람들이 길이 메워지도록 모두 나와서 우러러 전송하며 탄식하고 그분을 위해 눈물을 흘렸고, 또 그분을 위해 초상화를 그려서 사원(寺院)에 안치하고 제사를 지내고 있다. ”라고 말하였으므로, 이에 공(公)이 상주(常州) 사람들에게 은혜를 입히고 사랑을 베풀었음을 더욱 잘 알게 되었다. 그 후 공(公)의 아드님 처후(處厚)와 교유하게 되어 공(公)이 한 일을 매우 자세히 알게 되었다. 대체로 공(公)이 정사(政事)를 베풀 때에 정밀하고 분명하며 꿋꿋하고 과단성이 있어서, 일의 처리에 이르러서는 단안(斷案)을 내려서 적의(適宜)함을 얻었고, 오랫동안 간사(奸邪)한 짓을 하거나 악독한 짓을 한 사람은 곧 잡아들여 용서 없이 벌을 주었으며, 백성들이 감화하여 순복함에 이르러서는 그들의 뜻에 맞게 안무(按撫)하고 길러주어, 모두가 안주(安住)할 곳이 있게 하였다. 이에 원근(遠近)에 위엄이 크게 떨치게 되었고, 그의 은덕을 입은 사람들이 또한 그를 무궁토록 그리워하게 되었다. 명숙태후(明肅太后)께서 수렴청정(垂簾聽政)할 때를 당하여, 일찍이 공(公)을 등용하고자 한 일이 있었는데, 공(公)이 거듭 상서(上書)하여 당시(當時)의 국사(國事)를 논하면서 그 말에 직언(直言)을 한 것이 매우 많았으므로, 이 때문에 공(公)의 임용이 실현되지 못하고 상주지사(常州知事)로 나가게 되었던 것이다.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>당송팔대가문초증공1</t>
+          <t>당송팔대가문초왕안석2</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>251</v>
+        <v>434</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>考之於古則非訓이요 稽之於今則非利며 尋其名而求其實則失其宜라 故曰 議罷齋郞而以學生薦享이 亦不得其理矣라</t>
+          <t>吾友深父는 書足以致其言하고 言足以遂其志하며 志欲以聖人之道爲己任하야 蓋非至於命이면 弗止也라 故不爲小廉曲謹하야 以投衆人耳目하고 而取舍進退去就를 必度於仁義라 世皆稱其學問文章行治나 然眞知其人者不多요 而多見謂迂闊하야 不足趣時合變하니 嗟乎라 是乃所以爲深父也니 令深父而有以合乎彼면 則必無以同乎此矣리라</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>옛 제도를 상고해보면 교훈에 맞지 않고, 지금의 형편을 상고해보면 이롭지 않으며, 그 이름［名］과 실상［實］을 찾아보면 마땅함을 잃었다. 그러므로 “재랑(齋郞)을 없애고 학생에게 제향을 올리게 하자. ”는 논의 또한 사리(事理)에 맞지 않는다.</t>
+          <t>나의 친구 심보(深父)는, 글은 그의 말을 표현하기에 족(足)하고, 말은 그의 의지를 이루기에 족하였으며, 의지는 성인(聖人)의 도(道)를 자신의 임무로 삼아 천명(天命)을 아는 데 미치지 않으면 중지하고자 하지 않았다. 그러므로 소소한 청렴(淸廉)이나 세세한 일에 삼가는 것 따위로 중인(衆人)의 이목(耳目)을 끄는 일은 하려 하지 않았고, 취사(取捨)․진퇴(進退)․거취(去就)에 반드시 인의(仁義)를 기준으로 삼았다. 세상 사람들이 모두 그의 학문과 문장과 재능과 처신을 칭찬하였지만, 그의 인물됨을 제대로 아는 사람은 많지 않았고, 많은 이들에게 우활(迂闊)해서 시속(時俗)에 맞추어 임기응변을 하지 못하는 사람으로 인식되었다. 아아! 바로 이 점이 심보(深父)의 됨됨이의 근본이니, 심보(深父)로 하여금 저들에게 영합하는 일이 있게 하였다면, 반드시 이와 같게 될 수가 없었을 것이다.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>당송팔대가문초한유2</t>
+          <t>당송팔대가문초왕안석2</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>318</v>
+        <v>112</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>始吾讀孟軻書然後에 知孔子之道尊하고 聖人之道易行하고 王易王하고 霸易霸也로라 以爲孔子之徒沒에 尊聖人者는 孟氏而已라 晩得楊雄書하고는 益尊信孟氏로라 因雄書而孟氏益尊하니 則雄者도 亦聖人之徒歟ㄴ저</t>
+          <t>富室은 貧之母也니 誠不可破壞라 然使其大倖而役於下는 則又不可니라 兄云懼富人流爲工商浮窳라하니 蓋甚急而不均이면 則有此耳라 若富者雖益賦라도 而其實輸當其十一이면 猶足安其堵하여 雖驅之不肯易也리라 檢之逾精이면 則下逾巧는 誠如兄之言이라 管子亦不欲以民産爲征이라 故有殺畜伐木之說하니라 今若非市井之征이면 則捨其産 而唯丁田之問이니 推以誠質하고 示以恩惠하며 嚴責吏以法이니라 如所陳一社一村之制를 遞以信相考면 安有不得其實이리오 不得其實이면 則一社一村之制도 亦不可行矣리라 是故乘弊政 必須一定制니 而後兄之說乃得行焉이니라 蒙之所見及此而已라 永州以僻隅로 少知人事라 兄之所代者는 誰耶아 理歟弊歟아 理則其說行矣어니와 若其弊也면 蒙之說其在可用之數乎인저</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>처음에 내가 맹가(孟軻)의 글을 읽은 뒤에 공자(孔子)의 도(道)가 존귀(尊貴)하고, 성인(聖人)의 도(道)가 행(行)하기 쉽고, 왕도(王道)는 왕업(王業)을 이루기가 쉽고, 패도(霸道)는 패업(霸業)을 이루기가 쉽다는 것을 알았다.  〈나는〉 공자(孔子)의 제자들이 세상을 떠난 뒤에 성인(聖人)(공자(孔子))을 존숭(尊崇)한 이로는 맹씨(孟氏)뿐이라고 생각하였다.  뒤에 양웅(楊雄)의 글을 읽고는 더욱 맹씨(孟氏)를 존신(尊信)하였다. 양웅(楊雄)의 글로 인해 맹씨(孟氏)의 위상이 더욱 높아졌으니, 그렇다면 양웅(楊雄) 또한 성인(聖人)의 문도(門徒)이다.</t>
+          <t>부유한 가구(家口)는 가난한 가구의 어머니이므로 파괴해선 안 됩니다. 그러나 그들로 하여금 너무 큰 요행을 얻게 하여 아랫사람들을 부리게 하는 것 또한 안 됩니다. 형은 부유한 사람이 공상업(工商業)으로 직업을 바꾸어 빈둥거리며 지낼까 두렵다고 하셨는데, 부자들에 대한 세금징수를 매우 급하게 하거나 공정하게 하지 않으면 이런 문제가 있을 것입니다. 만약 부자에게 비록 부세(賦稅)가 늘어나더라도 정말 소득의 10분의 1만 내도록 한다면 오히려 충분히 그 속에서 안주하고 〈공상업(工商業)으로〉 내몰더라도 본업(本業)을 바꾸려 하지 않을 것입니다. 관청에서 점검을 정밀하게 하면 할수록 아래의 부자가 세금을 도피하는 수법이 더욱 교묘해진다는 것은 참으로 형의 말씀이 맞습니다. 관자(管子) 역시 백성의 재산에 따라 징세하려고 하지 않았으므로 “가축을 죽이거나 나무를 베지 말게 하라. ”는 설이 있습니다. 지금 만약 시정(市井)의 상인(商人)에게 징세하지 않는다면 〈농가(農家)에 대해서도〉 그 재산에 따라 징세하는 것을 그만두고 오직 인구(人口)와 전답(田畓)을 따져 징세하여야 할 것이니, 백성을 성심(誠心)으로 대하고 〈이 방법이〉 혜택이 크다는 점을 알리는 한편 법률로 관리를 엄격하게 단속해야 합니다. 그러면서 형께서 말씀하신 것처럼 1사(社), 1촌(村)의 단위별로 실사(實査)하는 제도를 만들어 차례대로 확실하게 실사한다면, 어찌 실상을 파악하지 못하겠습니까. 실상을 파악하지 못한다면 1사(社), 1촌(村)의 제도 역시 시행할 수 없습니다. 그러므로 전임 수령의 부패한 정사를 이어받았을 경우에는 반드시 일정한 제도가 있어야 하니, 그래야만 형께서 말씀하신 방법이 시행될 수 있습니다. 저의 소견은 여기까지입니다. 영주(永州)는 구석진 곳이어서 바깥세상의 정황을 잘 모릅니다. 형의 전임자는 누구입니까? 잘 다스렸습니까, 부패하였습니까? 잘 다스렸다면 형께서 주장하신 설이 시행될 것이지만, 만약 부패하였다면 저의 건의가 어쩌면 채용될 수도 있을 것입니다.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>당송팔대가문초한유2</t>
+          <t>당송팔대가문초유종원1</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>40</v>
+        <v>85</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>元和初에 收拾俊賢할새 徵拜吏部員外郞하고 未幾에 爲職方郞中知制誥하니라 友人得罪斥逐後에 其家親知도 過門縮頸不敢視로되 公獨省問하고 爲計度論議하야 直其寃하니라 由是出爲峽州刺史라가 轉廬州하니라 未至에 丁母夫人憂하니라 服除에 又爲婺州하니라 時疫旱甚하야 人死亡且盡이러니 公至하야 多方救活하니라 天遂雨하고 疫定하야 比數年里閭完復하니라 制使出巡에 人塡道迎顯公德하니라 事具聞에 就加金紫하니라 轉蘇州하야 變其屋居以絶火延하고 隄松江路하야 害絶阻滯하니라 秋夏賦調에 自爲書與人以期하야 吏無及門而集하니 政成爲天下守之最하다</t>
+          <t>其人材旣衆하여 列于庶位는 則如棫樸之盛에 得而薪之라 其以爲使臣엔 則寵其往也하되 必以禮樂하여 使其光華皇皇於遠近하고 勞其來也엔 則旣知其功하고 又本其情而敍其勤하니라 其以爲將率엔 則於其行也에 旣送遣之하고 又識薇蕨之始生하되 而恐其歸時之晩하며 及其還也에 旣休息之하고 又追念其悄悄之憂하되 而及於僕夫之瘁하니라 當此之時하여 后妃之於內助에 又知臣下之勤勞하니 其憂思之深은 至於山脊石砠僕馬之間하고 而志意之一은 至於雖采卷耳라도 而心不在焉이라 蓋先王之世에 待天下士 其勤且詳如此라 故稱周之士也貴하고 又稱周之士也肆하며 而天保亦稱君能下下하여 以成其政하고 臣能歸美하여 以報其上이라하니라 其君臣上下 相與之際如此하니 可謂至矣라</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>원화(元和) 초년에 재덕(才德)이 뛰어난 인재(人才)를 모을 때에 공을 불러 이부원외랑(吏部員外郞)에 제수하였고, 얼마 되지 않아 직방낭중(職方郞中) 지제고(知制誥)에 임명하였다. 왕공의 벗이 죄를 얻어 축출된 뒤로는 그 집안의 친척이나 지인(知人)들도 그 집 앞을 지날 적이면 목을 움츠리고 감히 바라보지도 못하였는데, 왕공은 홀로 가서 형편과 안부를 물었으며, 벗을 위해 계획하고 논의하여 벗의 억울함을 풀어주었다. 이로 인해 외직(外職)으로 나가 협주자사(峽州刺史)가 되었다가 여주자사(廬州刺史)로 전직(轉職)되었는데, 부임하기 전에 모친상(母親喪)을 당하였다. 상기(喪期)를 마친 뒤에 또 무주자사(婺州刺史)에 임명되었다. 이때 역병(疫病)과 가뭄이 심하여 사람들이 거의 다 죽게 되었는데, 왕공은 부임하자마자 여러 방법으로 구활(救活)하였다. 드디어 비가 내리고 역병도 진정되어 몇 년 전에 비해 민간의 생활이 완전히 회복되었다. 황제의 사자(使者)가 순시(巡視)를 나오자, 사람들이 길을 가득 메울 정도로 많이 나와서 사자를 맞이해 왕공의 공덕(功德)을 칭송하였다. 사자가 이 일을 구체적으로 아뢰니, 황제께서는 즉시 공에게 추가로 금자(金紫)의 관위(官位)를 내리셨다.  소주자사(蘇州刺史)로 옮겨가서는 가옥(家屋)의 형태를 변경하여 불이 번지는 것을 끊고, 송강(松江)에 제방을 쌓아 길을 만들어서 길이 막혀 생기는 피해를 없앴다. 가을과 여름에 부세를 징수할 때에는 직접 문서를 만들어 사람들에게 기한을 정해주어, 관리(官吏)가 찾아가지 않아도 백성이 스스로 와서 바치게 하니,  정사(政事)의 성적이 천하의 자사(刺史) 중에 으뜸이었다.</t>
+          <t>그리하여 인재가 이미 많이 확보되어 조정 백관에 배치한 것은 마치 두릅나무가 무성하게 자라 땔감이 필요할 때 그것을 사용하는 경우와 같았습니다.  이들을 사신으로 삼을 때는 외국에 나가는 것을 영예롭게 해주되 반드시 예의와 음악으로 해주어 그 영광이 원근의 이목에 환히 빛나도록 하였으며, 임무를 마치고 돌아온 자를 위로할 때는 이미 그 공을 알아주고 더 나아가 그 애절한 정을 이해하면서 공적을 평정해주었습니다. 그리고 장수로 삼을 적에는 그가 떠날 때 이미 예물을 증정하고, 또 고사리 싹이 돋아나 떠나야 할 때가 된 것을 알고 보내면서도 돌아오는 날이 혹시 늦어지지나 않을까 염려하였으며, 그가 돌아왔을 때에는 이미 편히 쉬도록 하고 또 그가 국사를 위해 노심초사 걱정했던 충정을 추념(追念)하면서 함께 따라간 마부의 고달픔까지도 돌아보았습니다.  이 당시에 문왕(文王)을 내조하는 후비(后妃)까지도 신하의 노고를 알았으니, 그 근심 걱정이 깊은 정도는 높은 산, 돌산, 종, 말 등을 거론하는 데까지 이르렀고,  마음이 한결같기로는 비록 권이(卷耳)［점나도나물］를 캐더라도 마음은 나물에 있지 않고 국사를 위해 고생하고 있을 신하들을 걱정할 정도였습니다.  대체로 선왕(先王)의 세상에서 천하의 선비를 대할 적에 정성을 다하고 또 소홀함이 없게 하기를 이처럼 하였기 때문에 “주(周)나라 선비는 존귀하였다. ” 하고, 또 “주(周)나라 선비는 거리낌이 없었다. ”고 하였으며, 〈천보(天保)〉편에서 “군주는 능히 아랫사람에게 자신을 낮추어 이상적인 정사를 이루었고, 신하는 능히 미덕을 윗사람에게 돌려 그 군상(君上)의 은혜에 보답하였다. ”고 하였습니다.  그 당시에는 군주와 신하 위아래가 서로 돕고 어울리기를 이와 같이 하였으니, 성대하다고 말할 수 있겠습니다.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>당송팔대가문초한유3</t>
+          <t>당송팔대가문초증공1</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>16</v>
+        <v>295</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>若夫坐如尸하며 立如齊니라.</t>
+          <t>守令之於民에 近且重을 易知矣라 予嘗論今之守令컨대 有道而聞四方者는 不過數人이니 此數人者는 非特任守令也라 過此數人하여는 有千里者相接이로되 而無一賢守요 有百里者相環이로되 而無一賢令이라 至天子大臣이 嘗患其然하여는 則任奉法之吏하고 嚴刺察之科하여 以繩治之에 諸郡守縣令이 以罪不任職하여 或黜或罷者 相繼於外라 於是에 下詔書하여 擇廷臣하여 使各擧所知以任守令하니 是天子大臣愛國與民而重守令之意 可謂無不至矣라 而詔雖下나 擧者卒不聞하고 惟令或以舊制擧로 不偕循歲月而授라 每擧者有姓名을 得而視之하고 推考其材行能堪其擧者에 卒亦未見焉이라 擧者旣然矣니 則以余之所見聞으로 陰計其人之孰可擧者에 卒亦未見焉이라 猶恐余之愚且賤이 聞與見焉者少하여 不足以知天下之材也하여는 則求夫賢而有名位聞與見之博者하여 而從之問其人之孰可擧者에 卒亦未見焉이나 豈天下之人固可誣하고 而天固不生材於今哉아</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>앉아 있을 때에는 시동(尸童)이 〈신위(神位)에〉 앉아 있는 것처럼 하고, 서 있을 때에는 재계(齋戒)할 때처럼 해야 한다.</t>
+          <t>수령(守令)이 백성들에게 있어 가깝고도 중요하다는 사실은 알기 쉽다. 나는 오늘날의 수령들에 관해 일찍이 논해보았다. 이들 가운데 도덕이 몸에 배어 사방에 명성이 알려진 사람은 몇 사람에 지나지 않으니, 이 몇 사람은 그 능력이 수령직을 맡을 자격을 넘어선다. 이 몇 사람 외에 천 리 되는 지역을 맡은 자가 여기저기 깔려 있지만 누구 하나 어진 군수가 없으며, 백 리 되는 지역을 맡은 자가 꼬리를 물고 이어져 있지만 누구 하나 어진 현령이 없다. 천자와 대신들은 일찍이 이러한 현실에 대해 우려했다. 그리하여 법을 신봉하는 관리들을 임용하고 규찰하는 법을 엄격하게 적용하여 법률의 잣대로 그들을 치죄하자, 여러 군수와 현령들 가운데 죄 때문에 관직을 맡지 못하고 폐출되거나 파면된 이들이 지방에서 잇따라 나타나게 되었다. 이에 조서(詔書)를 내려 조정 대신을 골라 이들이 각자 자신이 알던 사람들을 천거하도록 하여 수령직을 맡게 했다. 이로 볼 때 천자와 대신들이 나라를 사랑하고 백성들과 함께하며 수령을 중시하는 뜻이 모두 다 지극하다 할 수 있을 것이다. 그러나 비록 조서(詔書)가 내려졌는데도 천거된 자가 있다는 말은 끝내 들리지 않았고, 오로지 현령만 간혹 기존의 제거(制擧)제도를 적용하고 재직한 연한과 이력에 따라 관직을 제수하지는 않는다. 매번 천거 대상자의 성명이 밝혀지면 그것을 보고 그의 재능과 행실이 천거를 받기에 충분한지를 따져보면 그런 자를 끝내 볼 수가 없다. 천거 대상자가 이미 그런 실정이기에 내가 보고 들을 사실을 근거로 그 사람들 중에 누가 천거할 만한 사람인지 속으로 헤아려보면 또한 끝내 그런 자를 볼 수가 없다. 우매하고 미천한 내가 문견이 적어 천하의 인재들을 충분히 알아보지 못할까 염려되기에,  현명하여 명망과 지위가 있고 문견의 범위가 넓은 자를 찾아가 지금 세상에 천거할 만한 자가 과연 누구이겠느냐고 물어보아도 끝내 그런 자를 볼 수가 없다. 그러나 어찌 천하 사람들을 무시할 수 있겠으며, 하늘이 과연 지금 세상에 인재를 내지 않았겠는가.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>예기집설대전1</t>
+          <t>당송팔대가문초증공1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>99</v>
+        <v>251</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>藍田呂氏가 曰호대 出必告하고 反必面은 受命於親而不敢專也요, 所遊를 必有常하며 所習을 必有業은 體親之愛而不敢貽其憂也며 恒言不稱老는 極子之慕而不忍忘也니라. 父母在而不敢有其身하니 如之何聞斯行諸아. 出入而無所受命이면 是는 遺親也니 親之愛子가 至矣라 所遊에 必欲其安하고 所習에 必欲其正이니 苟輕身而不自愛면 則非所以養其志也라. 君子之事親에 親雖老而不失乎孺子慕者는 愛親之至也라. 孟子가 曰호대 五十而慕를 吾於大舜에 見之矣라. 故로 髧彼兩髦가 爲孺子之飾이나 親見然後에 說之라. 苟常言而稱老면 則忘親而非慕也라.</t>
+          <t>考之於古則非訓이요 稽之於今則非利며 尋其名而求其實則失其宜라 故曰 議罷齋郞而以學生薦享이 亦不得其理矣라</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>남전여씨(藍田呂氏): 외출할 때에는 반드시 아뢰고 돌아와서는 반드시 얼굴을 뵈는 것은, 부모에게 지시를 받아서 하고 마음대로 하지 않는 것이다. 가는 곳에는 반드시 일정한 장소가 있으며, 학습에는 반드시 일정한 과업(課業)이 있는 것은 부모의 사랑을 체득(體得)하여 감히 근심을 끼치지 않는 것이고, 평소 말하는 사이에 늙었다고 말하지 않는 것은 부모를 사모하는 마음을 극진하게 하여 차마 부모를 잊지 못하는 것이다. 부모가 살아 계시면 감히 그 몸은 마음대로 하지 못하는 법인데 어떻게 옳은 일이라고 그대로 행할 수 있겠는가. 들고 나면서 지시를 받는 바가 없으면 이는 부모를 버린 것이다. 부모가 자식을 사랑하는 것이 지극하기 때문에 갈 때에는 반드시 그가 편안하기를 바라고 학습할 때에는 반드시 바르게 배우기를 바라는 것이니 진실로 몸을 가볍게 생각하여 자신을 사랑하지 않는다면 이는 부모의 뜻을 받드는 것이 아니다. 군자가 부모를 섬김에 비록 부모는 늙고 〈나는 장성했더라도〉 어린 아이 때의 〈부모를〉 그리워하는 마음을 잃지 않는 것은 지극히 부모를 사랑하는 것이다. 《맹자(孟子)》에 이르기를 “50세가 되어서도 부모를 그리워하는 마음을 가진 이를 나는 순임금에게서 보았다. ”고 하였다. 그러므로 두 갈래로 늘어뜨린 다팔머리는 어린아이들이나 하는 꾸밈이지만 부모는 이것을 보고나서야 기뻐하니, 〈자신이 늙었더라도〉 만약 평소에 늙었다고 말한다면 이는 부모를 잊은 것이며 그리워하는 태도가 아니다.</t>
+          <t>옛 제도를 상고해보면 교훈에 맞지 않고, 지금의 형편을 상고해보면 이롭지 않으며, 그 이름［名］과 실상［實］을 찾아보면 마땅함을 잃었다. 그러므로 “재랑(齋郞)을 없애고 학생에게 제향을 올리게 하자. ”는 논의 또한 사리(事理)에 맞지 않는다.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>예기집설대전1</t>
+          <t>당송팔대가문초한유2</t>
         </is>
       </c>
     </row>
@@ -1136,72 +1136,72 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>敬君賜라 故로 不敢棄核이니라.</t>
+          <t>始吾讀孟軻書然後에 知孔子之道尊하고 聖人之道易行하고 王易王하고 霸易霸也로라 以爲孔子之徒沒에 尊聖人者는 孟氏而已라 晩得楊雄書하고는 益尊信孟氏로라 因雄書而孟氏益尊하니 則雄者도 亦聖人之徒歟ㄴ저</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>임금께서 하사한 것을 공경하는 까닭에 감히 씨를 버리지 못하는 것이다.</t>
+          <t>처음에 내가 맹가(孟軻)의 글을 읽은 뒤에 공자(孔子)의 도(道)가 존귀(尊貴)하고, 성인(聖人)의 도(道)가 행(行)하기 쉽고, 왕도(王道)는 왕업(王業)을 이루기가 쉽고, 패도(霸道)는 패업(霸業)을 이루기가 쉽다는 것을 알았다.  〈나는〉 공자(孔子)의 제자들이 세상을 떠난 뒤에 성인(聖人)(공자(孔子))을 존숭(尊崇)한 이로는 맹씨(孟氏)뿐이라고 생각하였다.  뒤에 양웅(楊雄)의 글을 읽고는 더욱 맹씨(孟氏)를 존신(尊信)하였다. 양웅(楊雄)의 글로 인해 맹씨(孟氏)의 위상이 더욱 높아졌으니, 그렇다면 양웅(楊雄) 또한 성인(聖人)의 문도(門徒)이다.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>예기집설대전1</t>
+          <t>당송팔대가문초한유2</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>449</v>
+        <v>40</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>疏에 曰호대 兵車는 革路也니 尙武猛無推讓이라. 故로 不式하나니라. 武車는 亦革路也니, 取其建戈刃하야는 卽云兵車요, 取其威猛하야는 卽云武車也라. 旌은 車上旌旛也니, 尙威武라 故로 舒散若垂緌然이오, 玉金象木四路는 不用兵이라 故로 曰德車니 德美在內하야 不尙赫奕이라 故로 纏結其旌於竿也라.</t>
+          <t>元和初에 收拾俊賢할새 徵拜吏部員外郞하고 未幾에 爲職方郞中知制誥하니라 友人得罪斥逐後에 其家親知도 過門縮頸不敢視로되 公獨省問하고 爲計度論議하야 直其寃하니라 由是出爲峽州刺史라가 轉廬州하니라 未至에 丁母夫人憂하니라 服除에 又爲婺州하니라 時疫旱甚하야 人死亡且盡이러니 公至하야 多方救活하니라 天遂雨하고 疫定하야 比數年里閭完復하니라 制使出巡에 人塡道迎顯公德하니라 事具聞에 就加金紫하니라 轉蘇州하야 變其屋居以絶火延하고 隄松江路하야 害絶阻滯하니라 秋夏賦調에 自爲書與人以期하야 吏無及門而集하니 政成爲天下守之最하다</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>소(疏): 병거(兵車)는 혁로(革路)이니, 용맹을 숭상하여 사양하는 일이 없으므로 식(式)의 예를 하지 않는다. 무거(武車)도 혁로(革路)이다. 수레에 무기를 둔다는 측면에서 말할 때는 병거(兵車)라 하고, 용맹스럽다는 측면에서 말할 때는 무거(武車)라 한다. 정(旌)은 수레 위에 세우는 깃발이니, 위무(威武)를 자랑하기 위한 것이다. 그러므로 펼쳐서 늘어뜨려 놓는 것이다. 옥로(玉路)‧금로(金路)‧상로(象路)‧목로(木路) 네 가지의 수레는 병기를 쓰지 않는다. 그러므로 덕거(德車)라고 한다. 덕의 아름다움은 내재적인 것이라서 〈겉으로〉 빛나는 아름다움을 숭상하지 않는다. 그러므로 정(旌)을 깃대에 묶어두는 것이다.</t>
+          <t>원화(元和) 초년에 재덕(才德)이 뛰어난 인재(人才)를 모을 때에 공을 불러 이부원외랑(吏部員外郞)에 제수하였고, 얼마 되지 않아 직방낭중(職方郞中) 지제고(知制誥)에 임명하였다. 왕공의 벗이 죄를 얻어 축출된 뒤로는 그 집안의 친척이나 지인(知人)들도 그 집 앞을 지날 적이면 목을 움츠리고 감히 바라보지도 못하였는데, 왕공은 홀로 가서 형편과 안부를 물었으며, 벗을 위해 계획하고 논의하여 벗의 억울함을 풀어주었다. 이로 인해 외직(外職)으로 나가 협주자사(峽州刺史)가 되었다가 여주자사(廬州刺史)로 전직(轉職)되었는데, 부임하기 전에 모친상(母親喪)을 당하였다. 상기(喪期)를 마친 뒤에 또 무주자사(婺州刺史)에 임명되었다. 이때 역병(疫病)과 가뭄이 심하여 사람들이 거의 다 죽게 되었는데, 왕공은 부임하자마자 여러 방법으로 구활(救活)하였다. 드디어 비가 내리고 역병도 진정되어 몇 년 전에 비해 민간의 생활이 완전히 회복되었다. 황제의 사자(使者)가 순시(巡視)를 나오자, 사람들이 길을 가득 메울 정도로 많이 나와서 사자를 맞이해 왕공의 공덕(功德)을 칭송하였다. 사자가 이 일을 구체적으로 아뢰니, 황제께서는 즉시 공에게 추가로 금자(金紫)의 관위(官位)를 내리셨다.  소주자사(蘇州刺史)로 옮겨가서는 가옥(家屋)의 형태를 변경하여 불이 번지는 것을 끊고, 송강(松江)에 제방을 쌓아 길을 만들어서 길이 막혀 생기는 피해를 없앴다. 가을과 여름에 부세를 징수할 때에는 직접 문서를 만들어 사람들에게 기한을 정해주어, 관리(官吏)가 찾아가지 않아도 백성이 스스로 와서 바치게 하니,  정사(政事)의 성적이 천하의 자사(刺史) 중에 으뜸이었다.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>예기집설대전1</t>
+          <t>당송팔대가문초한유3</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>622</v>
+        <v>171</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>君拜大夫之辱하고 大夫拜士之辱은 皆謂初爲大夫요, 初爲士而來見也라. 此後朝見則有常禮矣라. 士相見禮에 士見國君에 君答拜者는 亦以其初爲士而敬之也라. 主人拜辱은 拜其先施也니, 此는 謂尊卑相等者라. 言同國則異國은 亦當然矣니라.</t>
+          <t>志特謹書官爵及死葬月日하고 而行誼는 則蘊藉銘中이라</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>임금은 대부가 방문해 준 데 대한 사의(謝意)로 절을 하고, 대부는 사(士)가 방문해 준 데 대한 사의(謝意)로 절을 하는 것은, 모두 처음으로 대부(大夫)가 되거나 사(士)가 되어서 방문했을 때의 경우를 말한다. 이후에 조정에서 보게 되면 상례(常禮)로 한다. 사상견례(士相見禮)에서 사(士)가 임금을 뵐 때에 임금이 답배(答拜)한다는 것은 또한 그가 처음으로 사(士)가 되었기 때문에 그를 공경하는 것이다. 주인이 〈객이〉 방문해 준 데 대하여 절하는 것은 〈객이〉 먼저 베푼 데 대하여 절하는 것이니, 이것은 존비(尊卑)가 서로 같은 경우를 말한 것이다. 같은 나라의 경우를 말하였으니 다른 나라의 경우도 또한 마땅히 그런 것이다.</t>
+          <t>묘지(墓誌)에는 다만 관작(官爵) 및 사망한 월일(月日)과 장사 지낸 월일만을 삼가 기록하였고, 행의(行誼)는 명문(銘文) 가운데에 함축(含蓄)하였다.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>예기집설대전1</t>
+          <t>당송팔대가문초한유3</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>680</v>
+        <v>16</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>未及期는 在期日之前也라. 郤地는 閑隙之地也라. 下言相見은 及期日也라. 遇有遇禮하고 會有會禮라.</t>
+          <t>若夫坐如尸하며 立如齊니라.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>정해진 기일이 되기 전이라는 것은 만나기로 되어 있는 날이 되기 이전이다. 극지(郤地)는 〈양국의〉 중간에 있는 비어 있는 지역이다. 아래에서 말한 상견은 정해진 기일에 만나는 것이다. 우(遇)에는 우례(遇禮)가 있고, 회(會)에는 회례(會禮)가 있다.</t>
+          <t>앉아 있을 때에는 시동(尸童)이 〈신위(神位)에〉 앉아 있는 것처럼 하고, 서 있을 때에는 재계(齋戒)할 때처럼 해야 한다.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1212,839 +1212,1239 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>181</v>
+        <v>99</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>彈琴而後食者는 蓋以和平之聲으로 散感傷之情也라</t>
+          <t>藍田呂氏가 曰호대 出必告하고 反必面은 受命於親而不敢專也요, 所遊를 必有常하며 所習을 必有業은 體親之愛而不敢貽其憂也며 恒言不稱老는 極子之慕而不忍忘也니라. 父母在而不敢有其身하니 如之何聞斯行諸아. 出入而無所受命이면 是는 遺親也니 親之愛子가 至矣라 所遊에 必欲其安하고 所習에 必欲其正이니 苟輕身而不自愛면 則非所以養其志也라. 君子之事親에 親雖老而不失乎孺子慕者는 愛親之至也라. 孟子가 曰호대 五十而慕를 吾於大舜에 見之矣라. 故로 髧彼兩髦가 爲孺子之飾이나 親見然後에 說之라. 苟常言而稱老면 則忘親而非慕也라.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">거문고를 탄 뒤에 잡수신 것은 아마도 화평(和平)한 소리로써 감회가 있어 상심(傷心)한 마음을 흩어버린 것인 듯싶다. </t>
+          <t>남전여씨(藍田呂氏): 외출할 때에는 반드시 아뢰고 돌아와서는 반드시 얼굴을 뵈는 것은, 부모에게 지시를 받아서 하고 마음대로 하지 않는 것이다. 가는 곳에는 반드시 일정한 장소가 있으며, 학습에는 반드시 일정한 과업(課業)이 있는 것은 부모의 사랑을 체득(體得)하여 감히 근심을 끼치지 않는 것이고, 평소 말하는 사이에 늙었다고 말하지 않는 것은 부모를 사모하는 마음을 극진하게 하여 차마 부모를 잊지 못하는 것이다. 부모가 살아 계시면 감히 그 몸은 마음대로 하지 못하는 법인데 어떻게 옳은 일이라고 그대로 행할 수 있겠는가. 들고 나면서 지시를 받는 바가 없으면 이는 부모를 버린 것이다. 부모가 자식을 사랑하는 것이 지극하기 때문에 갈 때에는 반드시 그가 편안하기를 바라고 학습할 때에는 반드시 바르게 배우기를 바라는 것이니 진실로 몸을 가볍게 생각하여 자신을 사랑하지 않는다면 이는 부모의 뜻을 받드는 것이 아니다. 군자가 부모를 섬김에 비록 부모는 늙고 〈나는 장성했더라도〉 어린 아이 때의 〈부모를〉 그리워하는 마음을 잃지 않는 것은 지극히 부모를 사랑하는 것이다. 《맹자(孟子)》에 이르기를 “50세가 되어서도 부모를 그리워하는 마음을 가진 이를 나는 순임금에게서 보았다. ”고 하였다. 그러므로 두 갈래로 늘어뜨린 다팔머리는 어린아이들이나 하는 꾸밈이지만 부모는 이것을 보고나서야 기뻐하니, 〈자신이 늙었더라도〉 만약 평소에 늙었다고 말한다면 이는 부모를 잊은 것이며 그리워하는 태도가 아니다.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>예기집설대전2</t>
+          <t>예기집설대전1</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>481</v>
+        <v>318</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>季武子는 魯大夫季孫夙也라 蟜固는 人姓名이라 點은 字가 晳이니 曾子父也라 武子寢疾之時에 蟜固適有齊衰之服이라 遂衣凶服而問疾하고 且曰 大夫之門에 不當釋凶服이요 惟君門에 乃說(탈)耳어늘 此禮將亡하니 我之凶服以來는 欲以救此將亡之禮也라한대 武子善之言失禮之顯著者는 人皆可知요 若失禮之微細者는 惟君子라야 乃能表明之也라하니라 武子執政에 人所尊畏어늘 固之爲此는 欲以易時人之觀瞻하야 據禮而行이니 武子雖憾이나 不得而罪之也라 若倚門而歌則非禮矣니 其亦狂之一端歟인저 記者蓋善蟜固之存禮하고 譏曾點之廢禮也라</t>
+          <t>敬君賜라 故로 不敢棄核이니라.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>계무자(季武子)는 노(魯)나라 대부(大夫) 계손숙(季孫夙)이다. 교고(蟜固)는 사람의 성명이다. 점(點)의 자(字)는 석(晳)으로, 증자(曾子)의 아버지이다. 무자(武子)가 병으로 누워있을 때 교고가 마침 자최(齊衰)의 상복(喪服)을 입던 중이었다. 그래서 마침내 흉복(凶服)(상복)을 입고 가서 문병을 하고, 또 말하기를 “대부(大夫)의 문에서는 마땅히 흉복을 벗지 않아야 하고 오직 임금의 문에서만 벗을 뿐인데, 이러한 예가 장차 없어지게 생겼으니, 내가 흉복을 입은 채로 온 것은 장차 없어지려는 예의를 구제하고자 해서이다. ”라고 하자,  무자(武子)가 그 말을 좋게 여겨 말하기를 “실례(失禮)가 뚜렷하게 드러나는 것은 사람들이 모두 알 수 있지만, 만약 실례가 미세한 경우에는 오직 군자(君子)라야 그것을 분명하게 드러낼 수 있다. ”고 하였다.  무자(武子)가 정권을 장악함에 사람들이 존경하고 두려워하였는데 교고가 이 짓을 한 것은 그렇게 함으로써 당시 사람들의 보고 듣는 것을 바꾸고 싶어서 예(禮)에 근거하여 실행한 것이니, 무자가 비록 유감스럽게 여겼지만 그를 죄줄 수는 없었다. 증점(曾點)이 문에 기대어 노래부른 것과 같은 것은 예가 아니니, 그 또한 광자(狂者)의 한 단면일 것이다. 기록한 사람은 교고가 예를 보존한 것을 좋게 여기고, 증점이 예를 폐기한 것을 기롱한 것이다.</t>
+          <t>임금께서 하사한 것을 공경하는 까닭에 감히 씨를 버리지 못하는 것이다.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>예기집설대전2</t>
+          <t>예기집설대전1</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>792</v>
+        <v>449</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>蒙袂는 以袂蒙面也요 輯屨는 輯斂其足이니 言困憊而行蹇也라 貿貿는 垂頭喪氣之貌라 嗟來食은 歎閔之而使來食也라 從은 就也라 微與는 猶言細故末節이니 謂嗟來之言이 雖不敬이나 然亦非大過라 故其嗟雖可去나 而謝焉則可食矣라</t>
+          <t>疏에 曰호대 兵車는 革路也니 尙武猛無推讓이라. 故로 不式하나니라. 武車는 亦革路也니, 取其建戈刃하야는 卽云兵車요, 取其威猛하야는 卽云武車也라. 旌은 車上旌旛也니, 尙威武라 故로 舒散若垂緌然이오, 玉金象木四路는 不用兵이라 故로 曰德車니 德美在內하야 不尙赫奕이라 故로 纏結其旌於竿也라.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>몽몌(蒙袂)는 소매로 얼굴을 가렸다는 뜻이고 집구(輯屨)는 그 발을 모둔다는 뜻이니, 피곤하고 고달파 비틀거리며 걷는다는 말이다. 무무(貿貿)는 고개를 떨구고 기운을 잃은 모양이다. 차래식(嗟來食)은 탄식하고 가엾게 여겨서 와서 먹도록 했다는 뜻이다. 종(從)은 나아간다는 뜻이다. 미여(微與)는 작은 일․사소한 일이라는 말과 같으니, 쯧쯧거리며 오라고 한 말이 비록 불경스럽지만 또한 큰 잘못이 아니기 때문에 쯧쯧거릴 때에는 비록 〈주는 음식을 거절하고〉 떠나갈 수 있지만 사과를 했다면 먹을 수가 있는 것이다.</t>
+          <t>소(疏): 병거(兵車)는 혁로(革路)이니, 용맹을 숭상하여 사양하는 일이 없으므로 식(式)의 예를 하지 않는다. 무거(武車)도 혁로(革路)이다. 수레에 무기를 둔다는 측면에서 말할 때는 병거(兵車)라 하고, 용맹스럽다는 측면에서 말할 때는 무거(武車)라 한다. 정(旌)은 수레 위에 세우는 깃발이니, 위무(威武)를 자랑하기 위한 것이다. 그러므로 펼쳐서 늘어뜨려 놓는 것이다. 옥로(玉路)‧금로(金路)‧상로(象路)‧목로(木路) 네 가지의 수레는 병기를 쓰지 않는다. 그러므로 덕거(德車)라고 한다. 덕의 아름다움은 내재적인 것이라서 〈겉으로〉 빛나는 아름다움을 숭상하지 않는다. 그러므로 정(旌)을 깃대에 묶어두는 것이다.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>예기집설대전2</t>
+          <t>예기집설대전1</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>86</v>
+        <v>622</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>凡雜祠祭, 因事乃書. 或有得失可法戒, 則特書之. ◑非正統, 用正統雜祠祭例.</t>
+          <t>君拜大夫之辱하고 大夫拜士之辱은 皆謂初爲大夫요, 初爲士而來見也라. 此後朝見則有常禮矣라. 士相見禮에 士見國君에 君答拜者는 亦以其初爲士而敬之也라. 主人拜辱은 拜其先施也니, 此는 謂尊卑相等者라. 言同國則異國은 亦當然矣니라.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>무릇 잡사제(雜祠祭)는 사안을 통해서만 기록하였다. 혹 득실(得失)을 법식(法式)과 경계(警戒)로 삼을 수 있는 것은 특별히 기록하였다. ◑비정통(非正統)은 정통(正統)의 잡사제(雜祠祭)의 범례(凡例)를 썼다.</t>
+          <t>임금은 대부가 방문해 준 데 대한 사의(謝意)로 절을 하고, 대부는 사(士)가 방문해 준 데 대한 사의(謝意)로 절을 하는 것은, 모두 처음으로 대부(大夫)가 되거나 사(士)가 되어서 방문했을 때의 경우를 말한다. 이후에 조정에서 보게 되면 상례(常禮)로 한다. 사상견례(士相見禮)에서 사(士)가 임금을 뵐 때에 임금이 답배(答拜)한다는 것은 또한 그가 처음으로 사(士)가 되었기 때문에 그를 공경하는 것이다. 주인이 〈객이〉 방문해 준 데 대하여 절하는 것은 〈객이〉 먼저 베푼 데 대하여 절하는 것이니, 이것은 존비(尊卑)가 서로 같은 경우를 말한 것이다. 같은 나라의 경우를 말하였으니 다른 나라의 경우도 또한 마땅히 그런 것이다.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>자치통감강목1</t>
+          <t>예기집설대전1</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>96</v>
+        <v>680</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>凡非正統, 書法同. 但不書還, 或當特書以見事實, 則曰還某. 幸下著其字.</t>
+          <t>未及期는 在期日之前也라. 郤地는 閑隙之地也라. 下言相見은 及期日也라. 遇有遇禮하고 會有會禮라.</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>무릇 비정통(非正統)도 서법(書法)은 같다. 단 ‘환(還)’을 쓰지 않았다. 혹 특별히 써서 사실을 나타낼 경우에는 ‘환모(還某)’라 하고, 행(幸)은 아래에 ‘기(其)’자를 붙였다.</t>
+          <t>정해진 기일이 되기 전이라는 것은 만나기로 되어 있는 날이 되기 이전이다. 극지(郤地)는 〈양국의〉 중간에 있는 비어 있는 지역이다. 아래에서 말한 상견은 정해진 기일에 만나는 것이다. 우(遇)에는 우례(遇禮)가 있고, 회(會)에는 회례(會禮)가 있다.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>자치통감강목1</t>
+          <t>예기집설대전1</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>73</v>
+        <v>181</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>楚遷于壽春하다</t>
+          <t>彈琴而後食者는 蓋以和平之聲으로 散感傷之情也라</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>초(楚)나라가 수춘(壽春)으로 천도하였다.</t>
+          <t xml:space="preserve">거문고를 탄 뒤에 잡수신 것은 아마도 화평(和平)한 소리로써 감회가 있어 상심(傷心)한 마음을 흩어버린 것인 듯싶다. </t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>자치통감강목2</t>
+          <t>예기집설대전2</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>365</v>
+        <v>481</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>徙魏王豹爲西魏王하고</t>
+          <t>季武子는 魯大夫季孫夙也라 蟜固는 人姓名이라 點은 字가 晳이니 曾子父也라 武子寢疾之時에 蟜固適有齊衰之服이라 遂衣凶服而問疾하고 且曰 大夫之門에 不當釋凶服이요 惟君門에 乃說(탈)耳어늘 此禮將亡하니 我之凶服以來는 欲以救此將亡之禮也라한대 武子善之言失禮之顯著者는 人皆可知요 若失禮之微細者는 惟君子라야 乃能表明之也라하니라 武子執政에 人所尊畏어늘 固之爲此는 欲以易時人之觀瞻하야 據禮而行이니 武子雖憾이나 不得而罪之也라 若倚門而歌則非禮矣니 其亦狂之一端歟인저 記者蓋善蟜固之存禮하고 譏曾點之廢禮也라</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>위왕(魏王) 표(豹)를 옮겨서 서위왕(西魏王)으로 삼고,</t>
+          <t>계무자(季武子)는 노(魯)나라 대부(大夫) 계손숙(季孫夙)이다. 교고(蟜固)는 사람의 성명이다. 점(點)의 자(字)는 석(晳)으로, 증자(曾子)의 아버지이다. 무자(武子)가 병으로 누워있을 때 교고가 마침 자최(齊衰)의 상복(喪服)을 입던 중이었다. 그래서 마침내 흉복(凶服)(상복)을 입고 가서 문병을 하고, 또 말하기를 “대부(大夫)의 문에서는 마땅히 흉복을 벗지 않아야 하고 오직 임금의 문에서만 벗을 뿐인데, 이러한 예가 장차 없어지게 생겼으니, 내가 흉복을 입은 채로 온 것은 장차 없어지려는 예의를 구제하고자 해서이다. ”라고 하자,  무자(武子)가 그 말을 좋게 여겨 말하기를 “실례(失禮)가 뚜렷하게 드러나는 것은 사람들이 모두 알 수 있지만, 만약 실례가 미세한 경우에는 오직 군자(君子)라야 그것을 분명하게 드러낼 수 있다. ”고 하였다.  무자(武子)가 정권을 장악함에 사람들이 존경하고 두려워하였는데 교고가 이 짓을 한 것은 그렇게 함으로써 당시 사람들의 보고 듣는 것을 바꾸고 싶어서 예(禮)에 근거하여 실행한 것이니, 무자가 비록 유감스럽게 여겼지만 그를 죄줄 수는 없었다. 증점(曾點)이 문에 기대어 노래부른 것과 같은 것은 예가 아니니, 그 또한 광자(狂者)의 한 단면일 것이다. 기록한 사람은 교고가 예를 보존한 것을 좋게 여기고, 증점이 예를 폐기한 것을 기롱한 것이다.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>자치통감강목2</t>
+          <t>예기집설대전2</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>92</v>
+        <v>792</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>置宗正官하다 宗正, 秦官, 掌親屬, 帝復置之.</t>
+          <t>蒙袂는 以袂蒙面也요 輯屨는 輯斂其足이니 言困憊而行蹇也라 貿貿는 垂頭喪氣之貌라 嗟來食은 歎閔之而使來食也라 從은 就也라 微與는 猶言細故末節이니 謂嗟來之言이 雖不敬이나 然亦非大過라 故其嗟雖可去나 而謝焉則可食矣라</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>종정관(宗正官)을 두었다. 종정(宗正)은 진(秦)나라의 관직으로 친속(親屬)(종친(宗親))을 담당하였는데, 황제가 다시 두었다.</t>
+          <t>몽몌(蒙袂)는 소매로 얼굴을 가렸다는 뜻이고 집구(輯屨)는 그 발을 모둔다는 뜻이니, 피곤하고 고달파 비틀거리며 걷는다는 말이다. 무무(貿貿)는 고개를 떨구고 기운을 잃은 모양이다. 차래식(嗟來食)은 탄식하고 가엾게 여겨서 와서 먹도록 했다는 뜻이다. 종(從)은 나아간다는 뜻이다. 미여(微與)는 작은 일․사소한 일이라는 말과 같으니, 쯧쯧거리며 오라고 한 말이 비록 불경스럽지만 또한 큰 잘못이 아니기 때문에 쯧쯧거릴 때에는 비록 〈주는 음식을 거절하고〉 떠나갈 수 있지만 사과를 했다면 먹을 수가 있는 것이다.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>자치통감강목3</t>
+          <t>예기집설대전2</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>168</v>
+        <v>86</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>立南武侯織하여 爲南海王하다 織, 粤之世也. 文穎曰 “高祖五年, 以象郡‧桂林‧南海‧長沙, 立吳芮爲長沙王. 象郡‧桂林‧南海屬尉佗, 佗未降, 遙奪以封芮耳. 後佗降漢, 十一年更立佗爲南越王, 自此, 王三郡, 芮惟得長沙‧桂陽耳. 今封織南海王, 復遙奪佗一郡, 織未得王之. ”</t>
+          <t>凡雜祠祭, 因事乃書. 或有得失可法戒, 則特書之. ◑非正統, 用正統雜祠祭例.</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>남무후(南武侯) 직(織)을 세워 남해왕(南海王)으로 삼았다. 직(織)은 월(粤)의 후예(後裔)이다. 문영(文穎)이 말하기를 “고조(高祖) 5년(B. C. 202)에 상군(象郡), 계림군(桂林郡), 남해군(南海郡), 장사군(長沙郡)에 오예(吳芮)를 세워 장사왕(長沙王)으로 삼았다. 상군, 계림군, 남해군은 위타(尉佗)(조타(趙佗))에게 속했는데 위타가 항복하지 않자, 멀리서 이들 지역을 빼앗아 오예를 봉(封)한 것이다. 뒤에 위타가 한(漢)나라에 항복하자, 11년에 위타를 다시 세워 남월왕(南越王)으로 삼으니, 이로부터 위타는 세 군(郡)에 왕 노릇 하였고, 오예는 오직 장사(長沙)와 계양(桂陽)만을 얻었을 뿐이었다. 이제 직(織)을 남해왕(南海王)으로 봉(封)하여 다시 위타의 한 군(郡)(남해군(南海郡))을 멀리서 빼앗았으나 직(織)이 왕 노릇을 할 수 없었다. ” 하였다.</t>
+          <t>무릇 잡사제(雜祠祭)는 사안을 통해서만 기록하였다. 혹 득실(得失)을 법식(法式)과 경계(警戒)로 삼을 수 있는 것은 특별히 기록하였다. ◑비정통(非正統)은 정통(正統)의 잡사제(雜祠祭)의 범례(凡例)를 썼다.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>자치통감강목3</t>
+          <t>자치통감강목1</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>455</v>
+        <v>96</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>丞相御史請定律曰 諸當髡者는 爲城旦, 舂하고 當黥, 髡者는 鉗爲城旦, 舂하고 當劓者는 笞三百하고 當斬左止者는 笞五百하고 斬右止와 及殺人先自告와 及吏坐受賕枉法과 守縣官財物而卽盜之를 已論而復有笞罪者는 皆棄市하고 爲城旦, 舂者는 各有歲數以免이라한대 制曰 可라하다 當黥髡者, 刑法志 “作當黥者髡. ” 止, 與趾同, 足也. 當斬右足者, 以其罪次重, 故從棄市也. 殺人先自告, 謂殺人而自首, 得免罪者也. 賕, 音求, 賂也. 吏受賕枉法, 謂受賂而曲公法者也. 守縣官財物而卽盜之, 卽律所謂主守自盜者也. 殺人害重, 受賕盜物, 贓汚之身, 故此三罪, 已被論名而又犯笞, 亦皆棄市也. 城旦‧舂, (蒲)［滿］三歲爲鬼薪‧白粲, 鬼薪‧白粲一歲, 爲隷臣妾, 隷臣妾一歲, 免爲庶人. 隷臣妾, (蒲)［滿］二歲爲司寇, 司寇一歲及作如司寇二歲, 皆免爲庶人.</t>
+          <t>凡非正統, 書法同. 但不書還, 或當特書以見事實, 則曰還某. 幸下著其字.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>승상(丞相)과 어사(御史)가 법률을 정할 것을 청하여 아뢰기를 “곤(髡)(머리 깎음)에 해당되는 자는 성단(城旦)과 방아를 찧게 하고, 경(黥)(자자함)과 곤(髡)에 해당되는 자는 재갈을 물려 성단(城旦)과 방아를 찧게 하고, 의(劓)(코를 벰)에 해당되는 자는 태형(笞刑) 300대를 치고, 참좌지(斬左止)(왼발을 벰)에 해당되는 자는 태형(笞刑) 500대를 치고, 참우지(斬右止)(오른발을 벰)와 사람을 죽이고 먼저 자수하여 죄를 면제받은 자와 관리로서 뇌물을 받고 법을 부정하게 적용한 자와 현관(縣官)(국가)의 재물(財物)을 맡고서 도둑질한 죄에 걸린 자를 이미 논죄(論罪)하였는데 다시 태형(笞刑)의 죄를 범하였을 경우에는 모두 기시(棄市)하고, 성단(城旦)과 방아를 찧는 경우에는 각각 복역하는 연수(年數)를 두어서 면죄시켜야 합니다. ” 하니, 제(制)하기를 “좋다. ” 하였다. “당경곤(當黥髡)”은 ≪한서(漢書)≫ 〈형법지(刑法志)〉에 “경(黥)(자자)에 해당되는 자는 머리를 깎았다. ”라고 되어 있다. 지(止)는 지(趾)와 같으니, 발이다. 오른발을 벰에 해당되는 자는 그 죄가 두 번째로 무겁기 때문에 기시(棄市)를 따른 것이다. “살인선자고(殺人先自告)”는 사람을 죽이고 먼저 자수하여 죄를 면제받은 자를 이른다. 구(賕)는 음이 구(求)이니 뇌물이다. “이수구왕법(吏受賕枉法)”은 관리가 뇌물을 받고서 공정한 법을 부정하게 적용함을 이르고, “수현관재물이즉도지(守縣官財物而卽盜之)(현관(縣官)의 재물(財物)을 맡고서 도둑질했다. )”는 바로 법률에 이른바 ‘맡아서 지키는 자가 스스로 도둑질했다. ’는 것이다. 사람을 죽인 것은 폐해가 심하고, 뇌물을 받는 것과 국가의 물건을 도둑질한 것은 장죄(贓罪)를 지은 더러운 몸이다. 그러므로 이 세 가지 죄는 이미 논죄하는 이름을 입었는데 또다시 태형(笞刑)을 범했으면 또한 모두 기시(棄市)하는 것이다. 성단(城旦)과 방아를 찧게 하는 데 복역한 지 만 3년이 되었으면 귀신(鬼薪)과 백찬(白粲)에 복역하게 하며, 1년 동안 귀신과 백찬에 복역하였으면 노비가 되게 하며, 노비를 1년 동안 하였으면 죄를 면하여 서인(庶人)이 되게 한다. 노비를 한 지 만 2년이 되었으면 사구(司寇)에 복역하게 하고, 1년 동안 사구에 복역하였거나 또는 사구처럼 2년 동안 부역하였으면 모두 죄를 면하여 서인(庶人)이 되게 한다.</t>
+          <t>무릇 비정통(非正統)도 서법(書法)은 같다. 단 ‘환(還)’을 쓰지 않았다. 혹 특별히 써서 사실을 나타낼 경우에는 ‘환모(還某)’라 하고, 행(幸)은 아래에 ‘기(其)’자를 붙였다.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>자치통감강목3</t>
+          <t>자치통감강목1</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>198</v>
+        <v>170</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>休屠王太子日磾 沒入官하여 輸黃門養馬러니 帝遊宴見馬할새 後宮滿側이라 日磾等數十人이 牽馬過殿下라가 莫不竊視호되 至日磾하여는 獨不敢하다 日磾長八尺二寸이요 容貌甚嚴하고 馬又肥好하니 上이 奇焉하여 卽日에 賜湯沐, 衣冠하여 拜爲馬監이라가 遷侍中, 駙馬都尉, 光祿大夫하여 甚信愛之라 貴戚이 多竊怨曰 陛下妄得一胡兒하여 反貴重之라호대 上이 愈厚焉하고 以休屠作金人하여 爲祭天主라 故로 賜日磾姓金氏하다 磾, 丁奚切. 黃門, 屬少府, 職任親近, 以供天子, 百物在焉. 游宴見馬, 言方於游宴之時, 而召閱諸馬. 視, 視宮人也. 長, 直亮切. 黃門, 有馬監‧狗監. 駙馬都尉, 帝所置, 駙, 副馬也. 非正駕車, 皆爲副馬. 一曰 “駙, 近也, 疾也. ” 光祿大夫, 本中大夫, 帝改其名.</t>
+          <t>凡簒賊之臣書死.</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>휴저왕(休屠王)의 태자(太子)인 일제(日磾)가 적몰(籍沒)되어 관청에 들어와서 황문(黃門)으로 실려와 말을 길렀는데, 황제가 유연(遊宴)하면서 말을 사열(査閱)할 적에 후궁(後宮)들이 곁에 가득하였다. 일제 등 수십 명은 말을 끌고 궁전 아래를 지나다가 궁녀들을 훔쳐보지 않는 자가 없었으나, 일제만은 홀로 감히 궁녀들을 훔쳐보지 않았다. 일제는 신장이 8척(尺) 2촌(寸)이고 용모가 매우 엄숙하였으며, 그가 기르는 말들이 또 살지고 아름다우니, 상(上)은 기특히 여겨서 당일에 탕목읍(湯沐邑)과 의관(衣冠)을 하사하고 마감(馬監)을 제수하였다가 시중(侍中)과 부마도위(駙馬都尉), 광록대부(光祿大夫)로 승진시켜, 그를 매우 신임하고 사랑하였다. 이에 귀척(貴戚)들이 대부분 속으로 원망하기를 “폐하께서 망령되이 한 오랑캐 아이를 얻어서 도리어 그를 귀중하게 여긴다. ”라고 하였으나, 상(上)은 더욱 그를 친애하였고, 휴도국(休屠國)에서는 금인(金人)을 만들어 하늘에 제사하는 의식을 받는 주체로 삼는다 하여 일제에게 김씨(金氏) 성(姓)을 하사하였다. 제(磾)는 정해(丁奚)의 절(切)이다. 황문(黃門)은 소부(少府)에 속하였으니, 직임이 천자(天子) 가까이에 있으면서 천자에게 물건을 공급하였으므로 온갖 물건이 다 있었다. ‘유연견마(遊宴見馬)’는 한창 놀고 잔치할 적에 여러 말을 불러 사열(査閱)함을 말한 것이다. 시(視)는 궁인(宮人)을 살펴보는 것이다. 장(長)(길이)은 직량(直亮)의 절(切)이다. 황문(黃門)에 마감(馬監)과 구감(狗監)이 있었다. 부마도위(駙馬都尉)는 황제(무제(武帝))가 설치한 것이니, 부(駙)는 부마(副馬)이다. 정식으로 수레에 멍에 하는 말이 아닌 것을 모두 부마(副馬)라 한다. 일설에 “부(駙)는 가까움이요 빠름이다. ” 하였다. 광록대부(光祿大夫)는 본래 중대부(中大夫)였는데, 황제가 그 이름을 고쳤다.</t>
+          <t>무릇 찬적(簒賊)한 신하는 ‘사(死)’라고 기록하였다.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>자치통감강목4</t>
+          <t>자치통감강목1</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>536</v>
+        <v>200</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>上이 耕于鉅定하고 還幸泰山하여 修封禪하고 祀明堂이러니 見群臣하고 乃言曰 朕이 卽位以來로 所爲狂悖하여 使天下愁苦하니 不可追悔라 自今으로 事有傷害百姓하고 糜費天下者를 悉罷之하라 田千秋曰 方士言神僊者甚衆이나 而無顯功하니 請皆罷斥遣之하노이다 上曰 大鴻臚言이 是也라하고 於是에 悉罷諸方士候神人者하다 是後에 上이 每對群臣에 自歎曏時愚惑하여 爲方士所欺하니 天下에 豈有僊人이리오 盡妖妄耳라 節食服藥이면 差可少病而已라하니라 地理志 “鉅定縣, 屬齊國. ” 斥, 逐也.</t>
+          <t>又曰 “凡正統之君, 廢爲王公而死者, 書卒. ”</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>상(上)이 거정(鉅定)에서 친경(親耕)을 하고 돌아오다가 태산(泰山)에 행차하여 봉(封)을 보수하고 명당(明堂)에서 제사하였는데, 여러 신하들을 만나보고 마침내 말하기를 “짐(朕)이 즉위한 이래로 미친 짓을 하고 도리(道理)에 어긋난 행동을 하여 천하 사람들로 하여금 근심하고 괴롭게 하였으니, 후회막급이다. 지금으로부터 백성들에게 상해(폐해)를 끼치고 천하에 재물을 낭비하는 일을 모두 파하라. ” 하였다. 전천추(田千秋)가 아뢰기를 “방사(方士)로서 신선술(神仙術)을 말하는 자들이 매우 많으나 드러난 효험이 없으니, 모두 파하여 쫓아보낼 것을 청합니다. ” 하였다. 상(上)은 말하기를 “대홍려(大鴻臚)의 말이 옳다. ” 하고, 이에 신인(神人)을 기다리는 여러 방사들을 모두 파하였다. 이 뒤에 상(上)은 매번 신하들을 대할 적에 스스로 탄식하기를 “지난번에 내가 어리석고 미혹되어서 방사들에게 속임을 당하였으니, 천하에 어찌 신선(神仙)이 있겠는가. 모두 요망한 말일 뿐이다. 먹는 것을 절제하고 약을 먹으면 다소 병을 덜 수 있을 것이다. ” 하였다. ≪한서(漢書)≫ 〈지리지(地理志)〉에 “거정현(鉅定縣)은 제국(齊國)에 속하였다. ” 하였다. 척(斥)은 축출하다는 뜻이다.</t>
+          <t>또 말하기를, “무릇 정통의 임금이 폐위되어 왕공(王公)으로 죽은 경우에는 졸(卒)이라고 썼다. ”라고 하였다.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>자치통감강목4</t>
+          <t>자치통감강목1</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>332</v>
+        <v>322</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>◑夏六月에 大疫하니 詔損膳하고 減樂府員하고 省苑馬하여 以振困乏하다 樂府員, 大凡八百二十九人, 武帝所立. 漢官儀 “牧師諸苑三十六所, 分置北邊‧西邊, 養馬三十萬匹. ”</t>
+          <t>趙成侯種元年이라</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>여름 6월에 큰 역병(疫病)이 유행하자, 조령(詔令)을 내려 황제의 음식을 줄이고 악부(樂府)의 악공(樂工) 인원을 줄이고 동산의 말을 줄여서 궁핍한 자들을 구휼하게 하였다. 악부(樂府)의 악공(樂工) 인원은 대체로 829명이니, 무제(武帝)가 처음 세운 것이다. ≪한관의(漢官儀)≫에 “말을 기르는 목사(牧師)가 있는 원(苑) 36개소를 북변(北邊)과 서변(西邊)에 나누어 설치하여 30만 필(匹)의 말을 길렀다. ” 하였다.</t>
+          <t>조(趙)나라 성후(成侯) 종(種) 원년이다.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>자치통감강목5</t>
+          <t>자치통감강목1</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>145</v>
+        <v>386</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>永有所言, 令尙書郞受之.</t>
+          <t>趙肅侯元年이라</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>곡영(谷永)이 말하는 것이 있으면 상서(尙書)의 낭관(郞官)으로 하여금 받아오게 한 것이다.</t>
+          <t>조(趙)나라 숙후(肅侯) 원년이다.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>자치통감강목6</t>
+          <t>자치통감강목1</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>303</v>
+        <v>73</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>通鑑, 曉下, 有臣雖圖上, 猶須口說, 然後可知十二字. 間, 讀曰閑, 言願於淸淨燕安閑暇時, 賜召見.</t>
+          <t>楚遷于壽春하다</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">≪자치통감(資治通鑑)≫에는 효(曉)자 아래에 “신수도상(臣雖圖上) 유수구설(猶須口說) 연후가지(然後可知)라는 열두 글자가 있다. 간(間)은 한(閑)으로 읽으니, 조용하고 한가한 틈에 불러 만나주시기를 원함을 말한 것이다. </t>
+          <t>초(楚)나라가 수춘(壽春)으로 천도하였다.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>자치통감강목6</t>
+          <t>자치통감강목2</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>341</v>
+        <v>365</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>慶忌爲國虎臣하니 匈奴ㆍ西域이 敬其威信하니라</t>
+          <t>徙魏王豹爲西魏王하고</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>신경기(辛慶忌)가 나라의 호신(虎臣)이 되니, 흉노(匈奴)와 서역(西域)이 그의 위엄과 신의를 공경하였다.</t>
+          <t>위왕(魏王) 표(豹)를 옮겨서 서위왕(西魏王)으로 삼고,</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>자치통감강목6</t>
+          <t>자치통감강목2</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>945</v>
+        <v>92</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>相, 去聲, 其名也.</t>
+          <t>置宗正官하다 宗正, 秦官, 掌親屬, 帝復置之.</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>상(相)은 거성(去聲)이니, 그의 이름이다.</t>
+          <t>종정관(宗正官)을 두었다. 종정(宗正)은 진(秦)나라의 관직으로 친속(親屬)(종친(宗親))을 담당하였는데, 황제가 다시 두었다.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>자치통감강목6</t>
+          <t>자치통감강목3</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>1184</v>
+        <v>168</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>尊孝宣廟爲中宗하고 孝元廟爲高宗하다</t>
+          <t>立南武侯織하여 爲南海王하다 織, 粤之世也. 文穎曰 “高祖五年, 以象郡‧桂林‧南海‧長沙, 立吳芮爲長沙王. 象郡‧桂林‧南海屬尉佗, 佗未降, 遙奪以封芮耳. 後佗降漢, 十一年更立佗爲南越王, 自此, 王三郡, 芮惟得長沙‧桂陽耳. 今封織南海王, 復遙奪佗一郡, 織未得王之. ”</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>효선황제(孝宣皇帝)의 사당을 높여 중종(中宗)이라 하고 효원황제(孝元皇帝)의 사당을 높여 고종(高宗)이라 하였다.</t>
+          <t>남무후(南武侯) 직(織)을 세워 남해왕(南海王)으로 삼았다. 직(織)은 월(粤)의 후예(後裔)이다. 문영(文穎)이 말하기를 “고조(高祖) 5년(B. C. 202)에 상군(象郡), 계림군(桂林郡), 남해군(南海郡), 장사군(長沙郡)에 오예(吳芮)를 세워 장사왕(長沙王)으로 삼았다. 상군, 계림군, 남해군은 위타(尉佗)(조타(趙佗))에게 속했는데 위타가 항복하지 않자, 멀리서 이들 지역을 빼앗아 오예를 봉(封)한 것이다. 뒤에 위타가 한(漢)나라에 항복하자, 11년에 위타를 다시 세워 남월왕(南越王)으로 삼으니, 이로부터 위타는 세 군(郡)에 왕 노릇 하였고, 오예는 오직 장사(長沙)와 계양(桂陽)만을 얻었을 뿐이었다. 이제 직(織)을 남해왕(南海王)으로 봉(封)하여 다시 위타의 한 군(郡)(남해군(南海郡))을 멀리서 빼앗았으나 직(織)이 왕 노릇을 할 수 없었다. ” 하였다.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>자치통감강목6</t>
+          <t>자치통감강목3</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>1365</v>
+        <v>455</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>冬에 雷하고 桐華하고 大雨雹하다</t>
+          <t>丞相御史請定律曰 諸當髡者는 爲城旦, 舂하고 當黥, 髡者는 鉗爲城旦, 舂하고 當劓者는 笞三百하고 當斬左止者는 笞五百하고 斬右止와 及殺人先自告와 及吏坐受賕枉法과 守縣官財物而卽盜之를 已論而復有笞罪者는 皆棄市하고 爲城旦, 舂者는 各有歲數以免이라한대 制曰 可라하다 當黥髡者, 刑法志 “作當黥者髡. ” 止, 與趾同, 足也. 當斬右足者, 以其罪次重, 故從棄市也. 殺人先自告, 謂殺人而自首, 得免罪者也. 賕, 音求, 賂也. 吏受賕枉法, 謂受賂而曲公法者也. 守縣官財物而卽盜之, 卽律所謂主守自盜者也. 殺人害重, 受賕盜物, 贓汚之身, 故此三罪, 已被論名而又犯笞, 亦皆棄市也. 城旦‧舂, (蒲)［滿］三歲爲鬼薪‧白粲, 鬼薪‧白粲一歲, 爲隷臣妾, 隷臣妾一歲, 免爲庶人. 隷臣妾, (蒲)［滿］二歲爲司寇, 司寇一歲及作如司寇二歲, 皆免爲庶人.</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>겨울에 우레가 치고 오동나무에 꽃이 피고 큰 우박이 내렸다.</t>
+          <t>승상(丞相)과 어사(御史)가 법률을 정할 것을 청하여 아뢰기를 “곤(髡)(머리 깎음)에 해당되는 자는 성단(城旦)과 방아를 찧게 하고, 경(黥)(자자함)과 곤(髡)에 해당되는 자는 재갈을 물려 성단(城旦)과 방아를 찧게 하고, 의(劓)(코를 벰)에 해당되는 자는 태형(笞刑) 300대를 치고, 참좌지(斬左止)(왼발을 벰)에 해당되는 자는 태형(笞刑) 500대를 치고, 참우지(斬右止)(오른발을 벰)와 사람을 죽이고 먼저 자수하여 죄를 면제받은 자와 관리로서 뇌물을 받고 법을 부정하게 적용한 자와 현관(縣官)(국가)의 재물(財物)을 맡고서 도둑질한 죄에 걸린 자를 이미 논죄(論罪)하였는데 다시 태형(笞刑)의 죄를 범하였을 경우에는 모두 기시(棄市)하고, 성단(城旦)과 방아를 찧는 경우에는 각각 복역하는 연수(年數)를 두어서 면죄시켜야 합니다. ” 하니, 제(制)하기를 “좋다. ” 하였다. “당경곤(當黥髡)”은 ≪한서(漢書)≫ 〈형법지(刑法志)〉에 “경(黥)(자자)에 해당되는 자는 머리를 깎았다. ”라고 되어 있다. 지(止)는 지(趾)와 같으니, 발이다. 오른발을 벰에 해당되는 자는 그 죄가 두 번째로 무겁기 때문에 기시(棄市)를 따른 것이다. “살인선자고(殺人先自告)”는 사람을 죽이고 먼저 자수하여 죄를 면제받은 자를 이른다. 구(賕)는 음이 구(求)이니 뇌물이다. “이수구왕법(吏受賕枉法)”은 관리가 뇌물을 받고서 공정한 법을 부정하게 적용함을 이르고, “수현관재물이즉도지(守縣官財物而卽盜之)(현관(縣官)의 재물(財物)을 맡고서 도둑질했다. )”는 바로 법률에 이른바 ‘맡아서 지키는 자가 스스로 도둑질했다. ’는 것이다. 사람을 죽인 것은 폐해가 심하고, 뇌물을 받는 것과 국가의 물건을 도둑질한 것은 장죄(贓罪)를 지은 더러운 몸이다. 그러므로 이 세 가지 죄는 이미 논죄하는 이름을 입었는데 또다시 태형(笞刑)을 범했으면 또한 모두 기시(棄市)하는 것이다. 성단(城旦)과 방아를 찧게 하는 데 복역한 지 만 3년이 되었으면 귀신(鬼薪)과 백찬(白粲)에 복역하게 하며, 1년 동안 귀신과 백찬에 복역하였으면 노비가 되게 하며, 노비를 1년 동안 하였으면 죄를 면하여 서인(庶人)이 되게 한다. 노비를 한 지 만 2년이 되었으면 사구(司寇)에 복역하게 하고, 1년 동안 사구에 복역하였거나 또는 사구처럼 2년 동안 부역하였으면 모두 죄를 면하여 서인(庶人)이 되게 한다.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>자치통감강목6</t>
+          <t>자치통감강목3</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>514</v>
+        <v>111</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>復徭役을 比豐沛라</t>
+          <t>冬에 定二千石不擧孝廉罪法하다</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>풍패(豐沛)의 예와 같이 요역(徭役)을 면제해준 것이다.</t>
+          <t>겨울에 이천석(二千石)이 효성스럽거나 청렴한 자를 천거하지 않으면 처벌하는 법을 제정하였다.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>자치통감강목7</t>
+          <t>자치통감강목4</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>542</v>
+        <v>198</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>隗囂降蜀하다</t>
+          <t>休屠王太子日磾 沒入官하여 輸黃門養馬러니 帝遊宴見馬할새 後宮滿側이라 日磾等數十人이 牽馬過殿下라가 莫不竊視호되 至日磾하여는 獨不敢하다 日磾長八尺二寸이요 容貌甚嚴하고 馬又肥好하니 上이 奇焉하여 卽日에 賜湯沐, 衣冠하여 拜爲馬監이라가 遷侍中, 駙馬都尉, 光祿大夫하여 甚信愛之라 貴戚이 多竊怨曰 陛下妄得一胡兒하여 反貴重之라호대 上이 愈厚焉하고 以休屠作金人하여 爲祭天主라 故로 賜日磾姓金氏하다 磾, 丁奚切. 黃門, 屬少府, 職任親近, 以供天子, 百物在焉. 游宴見馬, 言方於游宴之時, 而召閱諸馬. 視, 視宮人也. 長, 直亮切. 黃門, 有馬監‧狗監. 駙馬都尉, 帝所置, 駙, 副馬也. 非正駕車, 皆爲副馬. 一曰 “駙, 近也, 疾也. ” 光祿大夫, 本中大夫, 帝改其名.</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>외효(隗囂)가 촉(蜀)에 항복하였다.</t>
+          <t>휴저왕(休屠王)의 태자(太子)인 일제(日磾)가 적몰(籍沒)되어 관청에 들어와서 황문(黃門)으로 실려와 말을 길렀는데, 황제가 유연(遊宴)하면서 말을 사열(査閱)할 적에 후궁(後宮)들이 곁에 가득하였다. 일제 등 수십 명은 말을 끌고 궁전 아래를 지나다가 궁녀들을 훔쳐보지 않는 자가 없었으나, 일제만은 홀로 감히 궁녀들을 훔쳐보지 않았다. 일제는 신장이 8척(尺) 2촌(寸)이고 용모가 매우 엄숙하였으며, 그가 기르는 말들이 또 살지고 아름다우니, 상(上)은 기특히 여겨서 당일에 탕목읍(湯沐邑)과 의관(衣冠)을 하사하고 마감(馬監)을 제수하였다가 시중(侍中)과 부마도위(駙馬都尉), 광록대부(光祿大夫)로 승진시켜, 그를 매우 신임하고 사랑하였다. 이에 귀척(貴戚)들이 대부분 속으로 원망하기를 “폐하께서 망령되이 한 오랑캐 아이를 얻어서 도리어 그를 귀중하게 여긴다. ”라고 하였으나, 상(上)은 더욱 그를 친애하였고, 휴도국(休屠國)에서는 금인(金人)을 만들어 하늘에 제사하는 의식을 받는 주체로 삼는다 하여 일제에게 김씨(金氏) 성(姓)을 하사하였다. 제(磾)는 정해(丁奚)의 절(切)이다. 황문(黃門)은 소부(少府)에 속하였으니, 직임이 천자(天子) 가까이에 있으면서 천자에게 물건을 공급하였으므로 온갖 물건이 다 있었다. ‘유연견마(遊宴見馬)’는 한창 놀고 잔치할 적에 여러 말을 불러 사열(査閱)함을 말한 것이다. 시(視)는 궁인(宮人)을 살펴보는 것이다. 장(長)(길이)은 직량(直亮)의 절(切)이다. 황문(黃門)에 마감(馬監)과 구감(狗監)이 있었다. 부마도위(駙馬都尉)는 황제(무제(武帝))가 설치한 것이니, 부(駙)는 부마(副馬)이다. 정식으로 수레에 멍에 하는 말이 아닌 것을 모두 부마(副馬)라 한다. 일설에 “부(駙)는 가까움이요 빠름이다. ” 하였다. 광록대부(光祿大夫)는 본래 중대부(中大夫)였는데, 황제가 그 이름을 고쳤다.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>자치통감강목7</t>
+          <t>자치통감강목4</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>603</v>
+        <v>536</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>彭이 上劉隆爲南郡太守하고 自率輔威將軍臧宮과 驍騎將軍劉歆하여 長驅入江關하여 令軍中無得虜掠하니 所過에 百姓이 皆奉牛酒迎勞라 彭이 復讓不受하니 百姓大喜하여 爭開門降이러라 詔彭守益州牧하고 所下郡에 輒行太守事하고 彭若出界하면 卽以太守號로 付後將軍하여 選官屬守州中長吏케하다 彭이 到江州하여 以其城固糧多하여 難卒拔이라하여 留馮駿守之하고 自引兵하여 乘利直指墊江하여 攻破平曲하고 收其米數十萬石하다 吳漢이 留夷陵하여 裝露橈繼進하다</t>
+          <t>上이 耕于鉅定하고 還幸泰山하여 修封禪하고 祀明堂이러니 見群臣하고 乃言曰 朕이 卽位以來로 所爲狂悖하여 使天下愁苦하니 不可追悔라 自今으로 事有傷害百姓하고 糜費天下者를 悉罷之하라 田千秋曰 方士言神僊者甚衆이나 而無顯功하니 請皆罷斥遣之하노이다 上曰 大鴻臚言이 是也라하고 於是에 悉罷諸方士候神人者하다 是後에 上이 每對群臣에 自歎曏時愚惑하여 爲方士所欺하니 天下에 豈有僊人이리오 盡妖妄耳라 節食服藥이면 差可少病而已라하니라 地理志 “鉅定縣, 屬齊國. ” 斥, 逐也.</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>잠팽(岑彭)은 황제에게 아뢰어 유륭(劉隆)을 남군태수(南郡太守)로 삼고, 자신이 직접 보위장군(輔威將軍) 장궁(臧宮)과 효기장군(驍騎將軍) 유흠(劉歆)을 거느리고서 멀리 치달려 강관(江關)으로 들어갔다. 잠팽이 군중(軍中)에게 명하여 노략질을 못하게 하니, 지나가는 곳마다 백성들이 모두 기뻐하여 소고기와 술을 받들어 맞이해 위로하였다. 잠팽이 다시 사양하고 받지 않으니, 백성들이 크게 기뻐하여 다투어 성문을 열고 항복하였다. 황제는 조령(詔令)을 내려 잠팽을 수익주목(守益州牧)으로 삼고 항복시킨 군(郡)마다 곧바로 태수(太守)의 일을 대행하게 하고, 잠팽이 만약 경내를 나가게 되면 즉시 태수(太守)의 칭호를 뒤에 오는 장군(將軍)에게 맡기게 하였다. 그리고 잠팽에게 관속 중에서 선발하여 익주(益州) 장리(長吏)의 직무를 대행하게 하였다. 잠팽은 강주성(江州城)에 이른 다음,  성이 견고하고 군량이 많아서 대번에 함락하기 어렵다고 판단하여 풍준(馮駿)을 남겨두어 지키게 하고, 자신은 직접 군대를 이끌고 승리한 틈을 타서 곧바로 점강(墊江)으로 향해 평곡(平曲)을 공격하여 깨뜨리고 이곳의 쌀 수십만 석(石)을 거두었다. 오한(吳漢)은 이릉(夷陵)에 남아서 노요(露橈)(전선(戰船)의 일종)를 정비하고서 계속 전진하게 하였다.</t>
+          <t>상(上)이 거정(鉅定)에서 친경(親耕)을 하고 돌아오다가 태산(泰山)에 행차하여 봉(封)을 보수하고 명당(明堂)에서 제사하였는데, 여러 신하들을 만나보고 마침내 말하기를 “짐(朕)이 즉위한 이래로 미친 짓을 하고 도리(道理)에 어긋난 행동을 하여 천하 사람들로 하여금 근심하고 괴롭게 하였으니, 후회막급이다. 지금으로부터 백성들에게 상해(폐해)를 끼치고 천하에 재물을 낭비하는 일을 모두 파하라. ” 하였다. 전천추(田千秋)가 아뢰기를 “방사(方士)로서 신선술(神仙術)을 말하는 자들이 매우 많으나 드러난 효험이 없으니, 모두 파하여 쫓아보낼 것을 청합니다. ” 하였다. 상(上)은 말하기를 “대홍려(大鴻臚)의 말이 옳다. ” 하고, 이에 신인(神人)을 기다리는 여러 방사들을 모두 파하였다. 이 뒤에 상(上)은 매번 신하들을 대할 적에 스스로 탄식하기를 “지난번에 내가 어리석고 미혹되어서 방사들에게 속임을 당하였으니, 천하에 어찌 신선(神仙)이 있겠는가. 모두 요망한 말일 뿐이다. 먹는 것을 절제하고 약을 먹으면 다소 병을 덜 수 있을 것이다. ” 하였다. ≪한서(漢書)≫ 〈지리지(地理志)〉에 “거정현(鉅定縣)은 제국(齊國)에 속하였다. ” 하였다. 척(斥)은 축출하다는 뜻이다.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>자치통감강목7</t>
+          <t>자치통감강목4</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>685</v>
+        <v>332</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>三月에 葬衛宣公하다</t>
+          <t>◑夏六月에 大疫하니 詔損膳하고 減樂府員하고 省苑馬하여 以振困乏하다 樂府員, 大凡八百二十九人, 武帝所立. 漢官儀 “牧師諸苑三十六所, 分置北邊‧西邊, 養馬三十萬匹. ”</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>3월에 위선공(衛宣公)을 장사 지냈다.</t>
+          <t>여름 6월에 큰 역병(疫病)이 유행하자, 조령(詔令)을 내려 황제의 음식을 줄이고 악부(樂府)의 악공(樂工) 인원을 줄이고 동산의 말을 줄여서 궁핍한 자들을 구휼하게 하였다. 악부(樂府)의 악공(樂工) 인원은 대체로 829명이니, 무제(武帝)가 처음 세운 것이다. ≪한관의(漢官儀)≫에 “말을 기르는 목사(牧師)가 있는 원(苑) 36개소를 북변(北邊)과 서변(西邊)에 나누어 설치하여 30만 필(匹)의 말을 길렀다. ” 하였다.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>춘추좌씨전1</t>
+          <t>자치통감강목5</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>692</v>
+        <v>145</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>鄭人來請脩好하다</t>
+          <t>永有所言, 令尙書郞受之.</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>정인(鄭人)이 노(魯)나라로 와서 수호(修好)하기를 청하였다.</t>
+          <t>곡영(谷永)이 말하는 것이 있으면 상서(尙書)의 낭관(郞官)으로 하여금 받아오게 한 것이다.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>춘추좌씨전1</t>
+          <t>자치통감강목6</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>708</v>
+        <v>303</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>許叔入于許하다</t>
+          <t>通鑑, 曉下, 有臣雖圖上, 猶須口說, 然後可知十二字. 間, 讀曰閑, 言願於淸淨燕安閑暇時, 賜召見.</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>허숙(許叔)이 허(許)로 들어갔다.</t>
+          <t xml:space="preserve">≪자치통감(資治通鑑)≫에는 효(曉)자 아래에 “신수도상(臣雖圖上) 유수구설(猶須口說) 연후가지(然後可知)라는 열두 글자가 있다. 간(間)은 한(閑)으로 읽으니, 조용하고 한가한 틈에 불러 만나주시기를 원함을 말한 것이다. </t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>춘추좌씨전1</t>
+          <t>자치통감강목6</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>822</v>
+        <v>341</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>夏에 衛侯入하야 放公子黔牟于周하고 放寗跪于秦하고 殺左公子洩右公子職하고 乃卽位하다</t>
+          <t>慶忌爲國虎臣하니 匈奴ㆍ西域이 敬其威信하니라</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>여름에 위후(衛侯)가 들어와서 공자(公子) 검모(黔牟)를 주(周)나라로, 영궤(甯跪)를 진(秦)나라로 추방하고 좌공자(左公子) 설(洩)과 우공자(右公子) 직(職)을 죽이고서 즉위하였다.</t>
+          <t>신경기(辛慶忌)가 나라의 호신(虎臣)이 되니, 흉노(匈奴)와 서역(西域)이 그의 위엄과 신의를 공경하였다.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>춘추좌씨전1</t>
+          <t>자치통감강목6</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>224</v>
+        <v>738</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>冬十有二月에 公會齊侯宋公陳侯衛侯鄭伯許男邢侯曹伯于淮하다</t>
+          <t>詔合葬共皇園하다</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>겨울 12월에 희공(僖公)이 제후(齊侯)‧송공(宋公)‧진후(陳侯)‧위후(衛侯)‧정백(鄭伯)‧허남(許男)‧형후(邢侯)‧조백(曹伯)과 회(淮)에서 회합(會合)하였다.</t>
+          <t>조령(詔令)을 내려서 공황(共皇)의 정도원(定陶園)에 합장하게 하였다.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>춘추좌씨전2</t>
+          <t>자치통감강목6</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>575</v>
+        <v>945</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>冬에 成風薨하다</t>
+          <t>相, 去聲, 其名也.</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>겨울에 성풍(成風)이 훙(薨)하였다.</t>
+          <t>상(相)은 거성(去聲)이니, 그의 이름이다.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>춘추좌씨전2</t>
+          <t>자치통감강목6</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>587</v>
+        <v>1184</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>六年春에 葬許僖公하다</t>
+          <t>尊孝宣廟爲中宗하고 孝元廟爲高宗하다</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>6년 봄에 허희공(許僖公)을 장사 지냈다.</t>
+          <t>효선황제(孝宣皇帝)의 사당을 높여 중종(中宗)이라 하고 효원황제(孝元皇帝)의 사당을 높여 고종(高宗)이라 하였다.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>춘추좌씨전2</t>
+          <t>자치통감강목6</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>406</v>
+        <v>1365</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>十有二月己丑에 公會晉侯齊侯宋公衛侯鄭伯曹伯邾子杞伯同盟于蟲牢하다</t>
+          <t>冬에 雷하고 桐華하고 大雨雹하다</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>12월 기축일(己丑日)에 성공(成公)이 진후(晉侯)‧제후(齊侯)‧송공(宋公)‧위후(衛侯)‧정백(鄭伯)‧조백(曹伯)‧주자(邾子)‧기백(杞伯)과 회합(會合)하여 충뢰(蟲牢)에서 동맹(同盟)하였다.</t>
+          <t>겨울에 우레가 치고 오동나무에 꽃이 피고 큰 우박이 내렸다.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>춘추좌씨전3</t>
+          <t>자치통감강목6</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>459</v>
+        <v>279</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>夏에 宋公使公孫壽來納幣하다</t>
+          <t>朱鮪殺李軼하고 攻溫, 平陰이어늘 馮異, 寇恂이 擊破之하다</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>여름에 송공(宋公)이 공손(公孫) 수(壽)를 보내 와서 납폐(納幣)하였다.</t>
+          <t>주유(朱鮪)가 이일(李軼)을 죽이고 온(溫)과 평음(平陰)을 공격하자, 풍이(馮異)와 구순(寇恂)이 격파하였다.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>춘추좌씨전3</t>
+          <t>자치통감강목7</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>623</v>
+        <v>514</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>戰之日에 齊國佐高無咎至于師하고 衛侯出于衛하고 公出于壞隤하다 宣伯通於穆姜하고 欲去季孟而取其室하다 將行에 穆姜送公할새 而使逐二子하니 公以晉難告 曰 請反而聽命이라하니 姜怒하다 公子偃公子鉏趨過러니 指之曰 女不可면 是皆君也라 公待於壞隤하야 申宮儆備하고 設守而後行하다 是以後하다 使孟獻子守于公宮하다</t>
+          <t>復徭役을 比豐沛라</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>교전(交戰)이 있은 다음날, 제(齊)나라 국좌(國佐)와 고무구(高無咎)가 군대를 거느리고 진(晉)나라의 군중(軍中)에 이르고, 위후(衛侯)도 위(衛)나라에서 출발(出發)하고, 성공(成公)도 괴퇴(壞隤)에서 출발(出發)하였다. 선백(宣伯)이 목강(穆姜)과 사통(私通)하고서, 계문자(季文子)와 맹헌자(孟獻子)를 제거(除去)하고 그 가산(家産)을 취(取)하고자 하였다. 출발(出發)하려 할 때 목강(穆姜)이 성공(成公)을 전송(餞送)하며 두 사람을 축출(逐出)하라고 하니, 성공(成公)이 진난(晉難)을 고(告)하면서 “돌아와서 명(命)을 듣겠습니다. ”고 하니, 목강(穆姜)은 노(怒)하였다. 그때 공자(公子) 언(偃)과 공자(公子) 서(鉏)가 빠른 걸음으로 지나가니, 목강(穆姜)이 그들을 가리키며 “네가 내 말을 듣지 않는다면 저 아이들이 모두 임금이 될 수 있다. ”고 하였다. 성공(成公)은 괴퇴(壞隤)에서 기다리면서 공궁(公宮)의 경비(警備)를 당부하고, 수비(守備)를 설치(設置)한 뒤에 출발(出發)하였기 때문에 뒤늦게 도착(到着)한 것이다. 성공(成公)은 떠날 때 맹헌자(孟獻子)에게 공궁(公宮)을 지키게 하였다.</t>
+          <t>풍패(豐沛)의 예와 같이 요역(徭役)을 면제해준 것이다.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>춘추좌씨전3</t>
+          <t>자치통감강목7</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>130</v>
+        <v>542</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>小邾子來朝하다</t>
+          <t>隗囂降蜀하다</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>소주자(小邾子)가 와서 조현(朝見)하였다.</t>
+          <t>외효(隗囂)가 촉(蜀)에 항복하였다.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>춘추좌씨전4</t>
+          <t>자치통감강목7</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>24</v>
+        <v>603</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>秋七月에 齊侯鄭伯爲衛侯故如晉하다 晉侯兼享之할새 晉侯賦嘉樂하니 國景子相齊侯하야 賦蓼蕭하고 子展相鄭伯하야 賦緇衣한대 叔向命晉侯拜二君曰 寡君敢拜齊君之安我先君之宗祧也하고 敢拜鄭君之不貳也하노라 國子使晏平仲私於叔向曰 晉君宣其明德於諸侯하야 恤其患而補其闕하고 正其違而治其煩일새 所以爲盟主也어늘 今爲臣執君하니 若之何오 叔向告趙文子한대 文子以告晉侯하니 晉侯言衛侯之罪하야 使叔向告二君하다 國子賦轡之柔矣하고 子展賦將仲子兮하니 晉侯乃許歸衛侯하다</t>
+          <t>彭이 上劉隆爲南郡太守하고 自率輔威將軍臧宮과 驍騎將軍劉歆하여 長驅入江關하여 令軍中無得虜掠하니 所過에 百姓이 皆奉牛酒迎勞라 彭이 復讓不受하니 百姓大喜하여 爭開門降이러라 詔彭守益州牧하고 所下郡에 輒行太守事하고 彭若出界하면 卽以太守號로 付後將軍하여 選官屬守州中長吏케하다 彭이 到江州하여 以其城固糧多하여 難卒拔이라하여 留馮駿守之하고 自引兵하여 乘利直指墊江하여 攻破平曲하고 收其米數十萬石하다 吳漢이 留夷陵하여 裝露橈繼進하다</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>가을 7월에 제후(齊侯)와 정백(鄭伯)이 위후(衛侯)를 돕기 위해 진(晉)나라에 갔다. 진후(晉侯)가 연회(宴會)를 열어 두 임금을 함께 접대(接待)할 때 진후(晉侯)가 〈가락편(嘉樂篇)〉을 읊으니, 제후(齊侯)의 상례(相禮) 국경자(國景子)가 〈요소편(蓼蕭篇)〉을 읊고, 정백(鄭伯)의 상례(相禮) 자전(子展)이 〈 치의편(緇衣篇)〉을 읊었다. 그러자 숙향(叔向)이 진후(晉侯)에게 명(命)하여 두 임금에게 배사(拜謝)하게 하고서 말하기를 “과군(寡君)은 감히 제군(齊君)께서 우리 선군(先君)의 종묘(宗廟)를 편안하게 하신 것에 대해 배사(拜謝)하고, 정군(鄭君)께서 두마음을 품지 않는 것에 대해 배사(拜謝)한 것입니다. ”고 하였다. 국자(國子)가 안평중(晏平仲)을 보내어 숙향(叔向)에게 사사로이 “진군(晉君)께서 밝은 덕행(德行)을 제후(諸侯)에게 선양(宣揚)하여 환난(患難)을 구휼(救恤)하고 결점(缺點)을 보완(補完)하며 잘못을 바로잡고 번란(煩亂)을 다스려 주셨기 때문에 맹주(盟主)가 되신 것인데, 지금 신하(臣下)를 위해 임금을 잡았으니 어째서입니까? ”라고 말하게 하였다. 숙향(叔向)이 이 말을 조문자(趙文子)에게 고(告)하자, 문자(文子)가 이를 진후(晉侯)에게 고하니, 진후(晉侯)는 위후(衛侯)의 죄상(罪狀)을 말해 주면서 숙향(叔向)을 시켜 두 임금에게 고(告)하게 하였다. 그러자 국자(國子)가 〈비지유의편(轡之柔矣篇)〉을 읊고 자전(子展)이 〈장중자혜편(將仲子兮篇)〉을 읊으니, 진후(晉侯)는 위후(衛侯)의 귀국(歸國)을 허락하였다.</t>
+          <t>잠팽(岑彭)은 황제에게 아뢰어 유륭(劉隆)을 남군태수(南郡太守)로 삼고, 자신이 직접 보위장군(輔威將軍) 장궁(臧宮)과 효기장군(驍騎將軍) 유흠(劉歆)을 거느리고서 멀리 치달려 강관(江關)으로 들어갔다. 잠팽이 군중(軍中)에게 명하여 노략질을 못하게 하니, 지나가는 곳마다 백성들이 모두 기뻐하여 소고기와 술을 받들어 맞이해 위로하였다. 잠팽이 다시 사양하고 받지 않으니, 백성들이 크게 기뻐하여 다투어 성문을 열고 항복하였다. 황제는 조령(詔令)을 내려 잠팽을 수익주목(守益州牧)으로 삼고 항복시킨 군(郡)마다 곧바로 태수(太守)의 일을 대행하게 하고, 잠팽이 만약 경내를 나가게 되면 즉시 태수(太守)의 칭호를 뒤에 오는 장군(將軍)에게 맡기게 하였다. 그리고 잠팽에게 관속 중에서 선발하여 익주(益州) 장리(長吏)의 직무를 대행하게 하였다. 잠팽은 강주성(江州城)에 이른 다음,  성이 견고하고 군량이 많아서 대번에 함락하기 어렵다고 판단하여 풍준(馮駿)을 남겨두어 지키게 하고, 자신은 직접 군대를 이끌고 승리한 틈을 타서 곧바로 점강(墊江)으로 향해 평곡(平曲)을 공격하여 깨뜨리고 이곳의 쌀 수십만 석(石)을 거두었다. 오한(吳漢)은 이릉(夷陵)에 남아서 노요(露橈)(전선(戰船)의 일종)를 정비하고서 계속 전진하게 하였다.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>춘추좌씨전5</t>
+          <t>자치통감강목7</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>307</v>
+        <v>264</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>王使問禮於左師與子産한대 左師曰 小國習之를 大國用之니 敢不薦聞이릿가하고 獻公合諸侯之禮六하다 子産曰 小國共職이니 敢不薦守릿가하고 獻伯子男會公之禮六하다 君子謂 合左師善守先代하고 子産善相小國이라</t>
+          <t>晉 姬姓 侯爵 武王少子唐叔虞之後也 成王封叔虞於唐 始都於翼 唐叔子燮父爲晉侯 傳十世 至昭侯 昭侯封其父文侯之弟成師於曲沃 是爲桓叔 昭侯傳至哀侯 爲桓叔之孫武公所滅 武公徙居絳 景公又徙新田 鄂侯二年 始入春秋 定公三十一年 魯哀公十四年也 又六世 韓魏趙三分晉地 遷其君靖公俱酒爲家人</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>초왕(楚王)이 사람을 보내어 좌사(左師)와 자산(子産)에게 예(禮)를 묻자, 좌사(左師)는 “소국(小國)이 강습(講習)한 예(禮)를 대국(大國)이 사용하려 하시니 감히 들은 바를 말씀드리지 않겠습니까? ”라고 하고서 공(公)이 제후(諸侯)를 회합(會合)하는 예(禮) 여섯 가지를 진언(進言)하고, 자산(子産)은 “소국(小國)은 직무(職務)를 봉행(奉行)해야 하니 감히 지키는 직분(職分)을 말씀드리지 않겠습니까? ”라고 하고서, 백(伯)‧자(子)‧남(男)이 공(公)과 회합(會合)하는 예(禮) 여섯 가지를 진언(進言)하였다. 군자(君子)는 이에 대해 다음과 같이 논평(論評)하였다. “합좌사(合左師)는 선대(先代)의 예(禮)를 잘 지켰다고 할 수 있고, 자산(子産)은 소국(小國)을 잘 보좌(輔佐)하였다고 할 수 있다. ”</t>
+          <t>진(晉) 희성(姬姓)이고 후작(侯爵)으로 무왕(武王)의 소자(少子) 당(唐) 숙우(叔虞)의 후손이다. 성왕(成王)이 숙우(叔虞)를 당(唐)에 봉(封)하였다. 비로소 익(翼)에 도읍(都邑)하고서 당숙의 아들 섭보(燮父)가 진후(晉侯)가 되었다. 10세(世)를 전(傳)하여 소후(昭侯)에 이르러 소후(昭侯)가 그 아버지 문후(文侯)의 아우 성사(成師)를 곡옥(曲沃)에 봉(封)하였으니, 이가 환숙(桓叔)이다. 소후(昭侯)로부터 나라를 전(傳)하여 애후(哀侯)에 이르러 환숙의 손자 무공(武公)에게 멸망되었다. 무공(武公)이 강(絳)으로 옮겨 거주(居住)하였고, 경공(景公)이 또 신전(新田)으로 천도(遷都)하였다. 악후(鄂侯) 2년부터 춘추시대로 들어섰다. 정공(定公) 31년이 노애공(魯哀公) 14년이다. 이로부터 6세(世) 뒤에 한(韓)‧위(魏)‧조(趙)가 진(晉)나라 땅을 삼분(三分)해 각각 일분(一分)씩을 차지하고서 그 임금 정공(靖公) 구주(俱酒)를 〈해상(海上)으로 옮겨〉 서인(庶人)으로 만들었다.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>춘추좌씨전5</t>
+          <t>춘추좌씨전1</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>85</v>
+        <v>685</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>秋七月이라</t>
+          <t>三月에 葬衛宣公하다</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>가을 7월이다.</t>
+          <t>3월에 위선공(衛宣公)을 장사 지냈다.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>춘추좌씨전6</t>
+          <t>춘추좌씨전1</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>4</v>
+        <v>692</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>秋에 晉士鞅宋樂祁犂衛北宮喜曹人邾人滕人會于扈</t>
+          <t>鄭人來請脩好하다</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>가을에 진(晉)나라 사앙(士鞅)이 송(宋)나라 악기리(樂祁犂), 위(衛)나라 북궁희(北宮喜), 조인(曹人), 주인(邾人), 등인(滕人)과 호(扈)에서 회합(會合)하였다.</t>
+          <t>정인(鄭人)이 노(魯)나라로 와서 수호(修好)하기를 청하였다.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>춘추좌씨전7</t>
+          <t>춘추좌씨전1</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>129</v>
+        <v>708</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>夏四月이라</t>
+          <t>許叔入于許하다</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>여름 4월이다.</t>
+          <t>허숙(許叔)이 허(許)로 들어갔다.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>춘추좌씨전7</t>
+          <t>춘추좌씨전1</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>183</v>
+        <v>822</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>夏에 季孫斯仲孫何忌如晉하다</t>
+          <t>夏에 衛侯入하야 放公子黔牟于周하고 放寗跪于秦하고 殺左公子洩右公子職하고 乃卽位하다</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>여름에 계손사(季孫斯)와 중손하기(仲孫何忌)가 진(晉)나라에 갔다.</t>
+          <t>여름에 위후(衛侯)가 들어와서 공자(公子) 검모(黔牟)를 주(周)나라로, 영궤(甯跪)를 진(秦)나라로 추방하고 좌공자(左公子) 설(洩)과 우공자(右公子) 직(職)을 죽이고서 즉위하였다.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>춘추좌씨전7</t>
+          <t>춘추좌씨전1</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>409</v>
+        <v>224</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>甲戌에 將戰할새 郵無恤御簡子하고 衛大子爲右하다 登鐵上하야 望見鄭師衆하고 大子懼하야 自投于車下하니 子良授大子綏而乘之曰 婦人也라 簡子巡列曰 畢萬은 匹夫也로되 七戰皆獲하야 有馬百乘하고 死於牖下하니 群子勉之하라 死不在寇니라 繁羽御趙羅하고 宋勇爲右러니 羅無勇이어늘 麇之하다 吏詰之한대 御對曰 痁作而伏이라하다 衛大子禱曰 曾孫蒯聵는 敢昭告皇祖文王과 烈祖康叔과 文祖襄公하노이다 鄭勝亂從하니 晉午在難하야 不能治亂하고 使鞅討之하니 蒯聵不敢自佚하고 備持矛焉하니 敢告無絶筋하고 無折骨하며 無面傷하야 以集大事하야 無作三祖羞하소서 大命은 不敢請이어니와 佩玉은 不敢愛로소이다</t>
+          <t>冬十有二月에 公會齊侯宋公陳侯衛侯鄭伯許男邢侯曹伯于淮하다</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>갑술일(甲戌日)에 교전(交戰)하려 할 때 우무휼(郵無恤)이 조간자(趙簡子)의 병거(兵車)를 몰고 위(衛)나라 태자(太子)가 거우(車右)가 되었다. 철구(鐵丘) 위로 올라가서 정군(鄭軍)이 많은 것을 바라보고는 위태자(衛太子)는 겁이 나서 스스로 병거(兵車) 아래로 굴러떨어지니, 자량(子良)이 태자(太子)에게 손잡이 끈을 쥐여주고 병거에 오르게 하며 말하기를 “여자처럼 겁이 많으십니다. ”고 하였다. 간자(簡子)가 대열(隊列)을 순행(巡行)하며 말하기를 “필만(畢萬)은 평범한 사내였으되 일곱 차례의 전투에서 모두 적을 사로잡았고, 말 4백 필(匹)을 가진 〈부자(富者)가 되어 편안히 살다가〉 천수(天壽)를 누리고 죽었으니, 그대들은 노력하라. 〈용감하게 싸운다면 반드시〉 적의 손에 죽지 않을 것이다. ”고 하였다. 번우(繁羽)가 조라(趙羅)의 병거를 몰고 송용(宋勇)이 거우(車右)가 되었는데, 조라(趙羅)가 용기(勇氣)가 없자, 그를 병거 안에 묶어놓았다. 군리(軍吏)가 그 이유를 묻자, 어(御)가 “저분은 학질(瘧疾)이 발작하여 엎드려 있는 것이다. ”고 대답하였다. 위태자(衛太子)는 〈출전(出戰)하기에 앞서〉 아래와 같이 기도(祈禱)하였다. “증손(曾孫) 괴외(蒯聵)는 감히 황조문왕(皇祖文王)과 열조강숙(烈祖康叔)과 문조양공(文祖襄公)께 밝게 고(告)하나이다. 정(鄭)나라 승(勝)이 순리를 어지럽히니 진(晉)나라 오(午)는 화난(禍難) 중에 있어 난인(亂人)을 다스리지 못하고, 조앙(趙鞅)을 보내어 난인(亂人)을 토벌하게 하니, 저 괴외(蒯聵)도 감히 스스로 편안히 있을 수 없어서 창을 드는 거우(車右)가 되었으니, 감히 고(告)하건대 힘줄이 끊기거나 뼈가 부러지거나 얼굴을 다치거나 하는 화(禍)가 없이 대사(大事)를 성공하여 세 할아버님의 수치가 되지 않게 하소서. 대명(大命)(생명(生命))은 감히 청(請)하지 않겠습니다만 패옥(佩玉)은 감히 아끼지 않겠나이다. ”</t>
+          <t>겨울 12월에 희공(僖公)이 제후(齊侯)‧송공(宋公)‧진후(陳侯)‧위후(衛侯)‧정백(鄭伯)‧허남(許男)‧형후(邢侯)‧조백(曹伯)과 회(淮)에서 회합(會合)하였다.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>춘추좌씨전7</t>
+          <t>춘추좌씨전2</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>469</v>
+        <v>575</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>孔子曰 楚昭王知大道矣니 其不失國也宜哉ᄂ저 夏書曰 惟彼陶唐으로 帥彼天常하야 有此冀方이어늘 今失其行하고 亂其紀綱하야 乃滅而亡이라하고 又曰 允出玆在玆라하니라 由己니 率常可矣니라</t>
+          <t>冬에 成風薨하다</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>공자(孔子)가 다음과 같이 논평(論評)하였다. “초소왕(楚昭王)이 대도(大道)를 알았으니, 그가 나라를 잃지 않은 것은 당연하다. 〈하서(夏書)〉에 ‘저 도당(陶唐)(제요(帝堯))으로부터 저 하늘의 상도(常道)를 준순(遵循)하여 이 기주지방(冀州地方)을 소유(所有)하였는데, 이제 그 도(道)를 잃고 그 기강(紀綱)을 어지럽혀 이에 멸망(滅亡)하였다. ’고 하고, 또 ‘진실로 이런 일이 생기는 것은 나에게 달렸다. ’고 하였다. 모든 화복(禍福)은 자신의 행위(行爲)에서 유래(由來)하니 상도(常道)를 따라야 한다. ”</t>
+          <t>겨울에 성풍(成風)이 훙(薨)하였다.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>춘추좌씨전7</t>
+          <t>춘추좌씨전2</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
+        <v>587</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>六年春에 葬許僖公하다</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>6년 봄에 허희공(許僖公)을 장사 지냈다.</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>춘추좌씨전2</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>224</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>夏에 楚子伐宋하니 以其救蕭也라 君子曰 淸丘之盟은 唯宋可以免焉이로다</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>여름에 초자(楚子)가 송(宋)나라를 토벌(討伐)하였으니, 이는 송(宋)나라가 소국(蕭國)을 구원(救援)하였기 때문이다. 군자(君子)는 이에 대해 다음과 같이 논평(論評)하였다. “청구(淸丘)의 결맹(結盟)은 오직 송(宋)나라만이 비난(非難)을 면(免)할 수 있다. ”</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>춘추좌씨전3</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>406</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>十有二月己丑에 公會晉侯齊侯宋公衛侯鄭伯曹伯邾子杞伯同盟于蟲牢하다</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>12월 기축일(己丑日)에 성공(成公)이 진후(晉侯)‧제후(齊侯)‧송공(宋公)‧위후(衛侯)‧정백(鄭伯)‧조백(曹伯)‧주자(邾子)‧기백(杞伯)과 회합(會合)하여 충뢰(蟲牢)에서 동맹(同盟)하였다.</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>춘추좌씨전3</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>459</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>夏에 宋公使公孫壽來納幣하다</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>여름에 송공(宋公)이 공손(公孫) 수(壽)를 보내 와서 납폐(納幣)하였다.</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>춘추좌씨전3</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>604</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>公至自會하다</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>성공(成公)이 회합(會合)에서 돌아왔다.</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>춘추좌씨전3</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>623</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>戰之日에 齊國佐高無咎至于師하고 衛侯出于衛하고 公出于壞隤하다 宣伯通於穆姜하고 欲去季孟而取其室하다 將行에 穆姜送公할새 而使逐二子하니 公以晉難告 曰 請反而聽命이라하니 姜怒하다 公子偃公子鉏趨過러니 指之曰 女不可면 是皆君也라 公待於壞隤하야 申宮儆備하고 設守而後行하다 是以後하다 使孟獻子守于公宮하다</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>교전(交戰)이 있은 다음날, 제(齊)나라 국좌(國佐)와 고무구(高無咎)가 군대를 거느리고 진(晉)나라의 군중(軍中)에 이르고, 위후(衛侯)도 위(衛)나라에서 출발(出發)하고, 성공(成公)도 괴퇴(壞隤)에서 출발(出發)하였다. 선백(宣伯)이 목강(穆姜)과 사통(私通)하고서, 계문자(季文子)와 맹헌자(孟獻子)를 제거(除去)하고 그 가산(家産)을 취(取)하고자 하였다. 출발(出發)하려 할 때 목강(穆姜)이 성공(成公)을 전송(餞送)하며 두 사람을 축출(逐出)하라고 하니, 성공(成公)이 진난(晉難)을 고(告)하면서 “돌아와서 명(命)을 듣겠습니다. ”고 하니, 목강(穆姜)은 노(怒)하였다. 그때 공자(公子) 언(偃)과 공자(公子) 서(鉏)가 빠른 걸음으로 지나가니, 목강(穆姜)이 그들을 가리키며 “네가 내 말을 듣지 않는다면 저 아이들이 모두 임금이 될 수 있다. ”고 하였다. 성공(成公)은 괴퇴(壞隤)에서 기다리면서 공궁(公宮)의 경비(警備)를 당부하고, 수비(守備)를 설치(設置)한 뒤에 출발(出發)하였기 때문에 뒤늦게 도착(到着)한 것이다. 성공(成公)은 떠날 때 맹헌자(孟獻子)에게 공궁(公宮)을 지키게 하였다.</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>춘추좌씨전3</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>130</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>小邾子來朝하다</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>소주자(小邾子)가 와서 조현(朝見)하였다.</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>춘추좌씨전4</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>24</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>秋七月에 齊侯鄭伯爲衛侯故如晉하다 晉侯兼享之할새 晉侯賦嘉樂하니 國景子相齊侯하야 賦蓼蕭하고 子展相鄭伯하야 賦緇衣한대 叔向命晉侯拜二君曰 寡君敢拜齊君之安我先君之宗祧也하고 敢拜鄭君之不貳也하노라 國子使晏平仲私於叔向曰 晉君宣其明德於諸侯하야 恤其患而補其闕하고 正其違而治其煩일새 所以爲盟主也어늘 今爲臣執君하니 若之何오 叔向告趙文子한대 文子以告晉侯하니 晉侯言衛侯之罪하야 使叔向告二君하다 國子賦轡之柔矣하고 子展賦將仲子兮하니 晉侯乃許歸衛侯하다</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>가을 7월에 제후(齊侯)와 정백(鄭伯)이 위후(衛侯)를 돕기 위해 진(晉)나라에 갔다. 진후(晉侯)가 연회(宴會)를 열어 두 임금을 함께 접대(接待)할 때 진후(晉侯)가 〈가락편(嘉樂篇)〉을 읊으니, 제후(齊侯)의 상례(相禮) 국경자(國景子)가 〈요소편(蓼蕭篇)〉을 읊고, 정백(鄭伯)의 상례(相禮) 자전(子展)이 〈 치의편(緇衣篇)〉을 읊었다. 그러자 숙향(叔向)이 진후(晉侯)에게 명(命)하여 두 임금에게 배사(拜謝)하게 하고서 말하기를 “과군(寡君)은 감히 제군(齊君)께서 우리 선군(先君)의 종묘(宗廟)를 편안하게 하신 것에 대해 배사(拜謝)하고, 정군(鄭君)께서 두마음을 품지 않는 것에 대해 배사(拜謝)한 것입니다. ”고 하였다. 국자(國子)가 안평중(晏平仲)을 보내어 숙향(叔向)에게 사사로이 “진군(晉君)께서 밝은 덕행(德行)을 제후(諸侯)에게 선양(宣揚)하여 환난(患難)을 구휼(救恤)하고 결점(缺點)을 보완(補完)하며 잘못을 바로잡고 번란(煩亂)을 다스려 주셨기 때문에 맹주(盟主)가 되신 것인데, 지금 신하(臣下)를 위해 임금을 잡았으니 어째서입니까? ”라고 말하게 하였다. 숙향(叔向)이 이 말을 조문자(趙文子)에게 고(告)하자, 문자(文子)가 이를 진후(晉侯)에게 고하니, 진후(晉侯)는 위후(衛侯)의 죄상(罪狀)을 말해 주면서 숙향(叔向)을 시켜 두 임금에게 고(告)하게 하였다. 그러자 국자(國子)가 〈비지유의편(轡之柔矣篇)〉을 읊고 자전(子展)이 〈장중자혜편(將仲子兮篇)〉을 읊으니, 진후(晉侯)는 위후(衛侯)의 귀국(歸國)을 허락하였다.</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>춘추좌씨전5</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>43</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>齊慶封來聘하다 其車美하니 孟孫謂叔孫曰 慶季之車가 不亦美乎아 叔孫曰 豹聞之컨대 服美不稱이면 必以惡終이라하니 美車何爲오 叔孫與慶封食에 不敬이어늘 爲賦相鼠로되 亦不知也하다</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>제(齊)나라 경봉(慶封)이 와서 빙문(聘問)하였다. 그가 타고 온 수레가 매우 아름다우니, 맹손(孟孫)이 숙손(叔孫)에게 말하기를 “경계(慶季)의 수레가 아름답지 않은가? ”라고 하자, 숙손(叔孫)이 말하기를 “내가 듣건대 거복(車服)이 아름다워 그 신분(身分)에 맞지 않으면 반드시 악(惡)(재앙)으로 끝난다고 하니, 아름다운 수레가 무슨 소용이 있겠는가? ”라고 하였다. 숙손(叔孫)이 경봉(慶封)과 식사(食事)를 하는데 경봉(慶封)이 공경(恭敬)하지 않자, 숙손(叔孫)이 상서시(相鼠詩)를 읊었는데도 경봉(慶封)은 그 이유를 알지 못하였다.</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>춘추좌씨전5</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>307</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>王使問禮於左師與子産한대 左師曰 小國習之를 大國用之니 敢不薦聞이릿가하고 獻公合諸侯之禮六하다 子産曰 小國共職이니 敢不薦守릿가하고 獻伯子男會公之禮六하다 君子謂 合左師善守先代하고 子産善相小國이라</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>초왕(楚王)이 사람을 보내어 좌사(左師)와 자산(子産)에게 예(禮)를 묻자, 좌사(左師)는 “소국(小國)이 강습(講習)한 예(禮)를 대국(大國)이 사용하려 하시니 감히 들은 바를 말씀드리지 않겠습니까? ”라고 하고서 공(公)이 제후(諸侯)를 회합(會合)하는 예(禮) 여섯 가지를 진언(進言)하고, 자산(子産)은 “소국(小國)은 직무(職務)를 봉행(奉行)해야 하니 감히 지키는 직분(職分)을 말씀드리지 않겠습니까? ”라고 하고서, 백(伯)‧자(子)‧남(男)이 공(公)과 회합(會合)하는 예(禮) 여섯 가지를 진언(進言)하였다. 군자(君子)는 이에 대해 다음과 같이 논평(論評)하였다. “합좌사(合左師)는 선대(先代)의 예(禮)를 잘 지켰다고 할 수 있고, 자산(子産)은 소국(小國)을 잘 보좌(輔佐)하였다고 할 수 있다. ”</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>춘추좌씨전5</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>361</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>大夫如秦하야 葬景公하니 禮也라</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>대부(大夫)가 진(秦)나라에 가서 진경공(秦景公)을 장사(葬事) 지냈으니 예(禮)에 맞았다.</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>춘추좌씨전5</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>85</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>秋七月이라</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>가을 7월이다.</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>춘추좌씨전6</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>305</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>晉人圍郊하다</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>진인(晉人)이 교(郊)를 포위하였다.</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>춘추좌씨전6</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>4</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>秋에 晉士鞅宋樂祁犂衛北宮喜曹人邾人滕人會于扈</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>가을에 진(晉)나라 사앙(士鞅)이 송(宋)나라 악기리(樂祁犂), 위(衛)나라 북궁희(北宮喜), 조인(曹人), 주인(邾人), 등인(滕人)과 호(扈)에서 회합(會合)하였다.</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>춘추좌씨전7</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>129</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>夏四月이라</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>여름 4월이다.</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>춘추좌씨전7</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>183</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>夏에 季孫斯仲孫何忌如晉하다</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>여름에 계손사(季孫斯)와 중손하기(仲孫何忌)가 진(晉)나라에 갔다.</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>춘추좌씨전7</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>340</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>十有五年春王正月에 邾子來朝하다</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>15년 봄 주왕(周王) 정월(正月)에 주자(邾子)가 와서 조현(朝見)하였다.</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>춘추좌씨전7</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>409</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>甲戌에 將戰할새 郵無恤御簡子하고 衛大子爲右하다 登鐵上하야 望見鄭師衆하고 大子懼하야 自投于車下하니 子良授大子綏而乘之曰 婦人也라 簡子巡列曰 畢萬은 匹夫也로되 七戰皆獲하야 有馬百乘하고 死於牖下하니 群子勉之하라 死不在寇니라 繁羽御趙羅하고 宋勇爲右러니 羅無勇이어늘 麇之하다 吏詰之한대 御對曰 痁作而伏이라하다 衛大子禱曰 曾孫蒯聵는 敢昭告皇祖文王과 烈祖康叔과 文祖襄公하노이다 鄭勝亂從하니 晉午在難하야 不能治亂하고 使鞅討之하니 蒯聵不敢自佚하고 備持矛焉하니 敢告無絶筋하고 無折骨하며 無面傷하야 以集大事하야 無作三祖羞하소서 大命은 不敢請이어니와 佩玉은 不敢愛로소이다</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>갑술일(甲戌日)에 교전(交戰)하려 할 때 우무휼(郵無恤)이 조간자(趙簡子)의 병거(兵車)를 몰고 위(衛)나라 태자(太子)가 거우(車右)가 되었다. 철구(鐵丘) 위로 올라가서 정군(鄭軍)이 많은 것을 바라보고는 위태자(衛太子)는 겁이 나서 스스로 병거(兵車) 아래로 굴러떨어지니, 자량(子良)이 태자(太子)에게 손잡이 끈을 쥐여주고 병거에 오르게 하며 말하기를 “여자처럼 겁이 많으십니다. ”고 하였다. 간자(簡子)가 대열(隊列)을 순행(巡行)하며 말하기를 “필만(畢萬)은 평범한 사내였으되 일곱 차례의 전투에서 모두 적을 사로잡았고, 말 4백 필(匹)을 가진 〈부자(富者)가 되어 편안히 살다가〉 천수(天壽)를 누리고 죽었으니, 그대들은 노력하라. 〈용감하게 싸운다면 반드시〉 적의 손에 죽지 않을 것이다. ”고 하였다. 번우(繁羽)가 조라(趙羅)의 병거를 몰고 송용(宋勇)이 거우(車右)가 되었는데, 조라(趙羅)가 용기(勇氣)가 없자, 그를 병거 안에 묶어놓았다. 군리(軍吏)가 그 이유를 묻자, 어(御)가 “저분은 학질(瘧疾)이 발작하여 엎드려 있는 것이다. ”고 대답하였다. 위태자(衛太子)는 〈출전(出戰)하기에 앞서〉 아래와 같이 기도(祈禱)하였다. “증손(曾孫) 괴외(蒯聵)는 감히 황조문왕(皇祖文王)과 열조강숙(烈祖康叔)과 문조양공(文祖襄公)께 밝게 고(告)하나이다. 정(鄭)나라 승(勝)이 순리를 어지럽히니 진(晉)나라 오(午)는 화난(禍難) 중에 있어 난인(亂人)을 다스리지 못하고, 조앙(趙鞅)을 보내어 난인(亂人)을 토벌하게 하니, 저 괴외(蒯聵)도 감히 스스로 편안히 있을 수 없어서 창을 드는 거우(車右)가 되었으니, 감히 고(告)하건대 힘줄이 끊기거나 뼈가 부러지거나 얼굴을 다치거나 하는 화(禍)가 없이 대사(大事)를 성공하여 세 할아버님의 수치가 되지 않게 하소서. 대명(大命)(생명(生命))은 감히 청(請)하지 않겠습니다만 패옥(佩玉)은 감히 아끼지 않겠나이다. ”</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>춘추좌씨전7</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>423</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>夏五月辛卯에 司鐸火하야 火踰公宮하야 桓僖災하니 救火者皆曰 顧府하라하다 南宮敬叔至하야 命周人하야 出御書하야 俟於宮하고 曰 庀女하리니 而不在면 死하리라 子服景伯至하야 命宰人호되 出禮書하야 以待命하라 命不共이면 有常刑하리라 校人乘馬하고 巾車脂轄하며 百官官備하야 府庫愼守하고 官人肅給하라 濟濡帷幕하야 鬱攸從之하라 蒙葺公屋호되 自大廟始하야 外內以悛하고 助所不給하라 有不用命이면 則有常刑하니 無赦하리라 公父文伯至하야 命校人駕乘車하다 季桓子至하야 御公立于象魏之外하야 命救火者호되 傷人則止하라 財可爲也니라 命藏象魏曰 舊章不可亡也니라 富父槐至하야 曰 無備而官辦者는 猶拾瀋也라 於是乎去表之槀하고 道還公宮하다</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>여름 5월 신묘일(辛卯日)에 사탁(司鐸)에 화재(火災)가 발생하여 그 불이 공궁(公宮)으로 넘어와 환공(桓公)과 희공(僖公)의 묘(廟)를 태웠다. 이때 불을 끄는 자들은 모두 “부고(府庫)를 주의해 살피라. ”고 하였다. 남궁경숙(南宮敬叔)이 와서 주인(周人)에게 명(命)하여 어서(御書)를 구출(救出)하여 궁(宮)에서 기다리게 하고서 말하기를 “불이 잡힌 뒤에 너에게 이 어서(御書)를 챙겨 올리게 할 것이니, 그때 만약 손실(損失)된 것이 있으면 사죄(死罪)로 다스릴 것이다. ”고 하였다. 자복경백(子服景伯)이 와서 재인(宰人)에게 명하기를 “예서(禮書)를 구출(救出)하고서 명(命)을 기다리라. 명(命)을 받들지 않으면 정해진 법(法)에 따라 처벌(處罰)할 것이다. 교인(校人)은 수레에 메울 네 필의 말을 준비하고, 건거(巾車)는 수레바퀴에 기름을 치고, 백관(百官)들은 각자의 직무(職務)를 다하여, 〈부인(府人)과 고인(庫人)은〉 부고(府庫)를 조심해 지키고, 관인(官人)(관인(館人))은 엄숙히 공급(供給)하라. 유막(帷幕)을 물에 적셔 불이 붙을 만한 곳으로 가라. 공궁(公宮)의 지붕을 덮되 태묘(太廟)의 지붕부터 먼저 덮고, 밖과 안을 차례로 덮으라. 인력(人力)이 부족한 곳에는 인력(人力)을 보조(補助)하라. 명(命)을 따르지 않는 자가 있으면 정해진 법(法)에 따라 처벌하고 용서하지 않을 것이다. ”고 하였다. 공보문백(公父文伯)이 와서 교인(校人)에게 승거(乘車)(임금의 수레)에 말을 메우라고 명하였다. 계환자(季桓子)가 와서 애공(哀公)을 수레에 모시고서 상위(象魏) 밖에 서서 불을 끄는 사람들에게 명하기를 “불의 기세에 사람이 상(傷)할 성싶으면 불 끄는 일을 중지하라. 재물(財物)은 다시 모을 수 있다. ”고 하였다. 그리고 또 상위(象魏)를 갈무리하라고 명하며 말하기를 “옛 전장(典章)을 잃어서는 안 된다. ”고 하였다. 부부괴(富父槐)가 와서 말하기를 “화재의 대비가 없으면서 백관에게 책임을 지우는 것은 엎지른 국물을 수습하게 하는 것과 같다. ”고 하고서 이에 불길을 표시한 곳에 쌓인 마른 나무들을 다 제거하고, 공궁(公宮) 둘레의 길을 깨끗이 치웠다.</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>춘추좌씨전7</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>469</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>孔子曰 楚昭王知大道矣니 其不失國也宜哉ᄂ저 夏書曰 惟彼陶唐으로 帥彼天常하야 有此冀方이어늘 今失其行하고 亂其紀綱하야 乃滅而亡이라하고 又曰 允出玆在玆라하니라 由己니 率常可矣니라</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>공자(孔子)가 다음과 같이 논평(論評)하였다. “초소왕(楚昭王)이 대도(大道)를 알았으니, 그가 나라를 잃지 않은 것은 당연하다. 〈하서(夏書)〉에 ‘저 도당(陶唐)(제요(帝堯))으로부터 저 하늘의 상도(常道)를 준순(遵循)하여 이 기주지방(冀州地方)을 소유(所有)하였는데, 이제 그 도(道)를 잃고 그 기강(紀綱)을 어지럽혀 이에 멸망(滅亡)하였다. ’고 하고, 또 ‘진실로 이런 일이 생기는 것은 나에게 달렸다. ’고 하였다. 모든 화복(禍福)은 자신의 행위(行爲)에서 유래(由來)하니 상도(常道)를 따라야 한다. ”</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>춘추좌씨전7</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
         <v>44</v>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B101" t="inlineStr">
         <is>
           <t>衛孔圉取大子蒯聵之姊하야 生悝하다 孔氏之豎渾良夫長而美러니 孔文子卒에 通于內하다 大子在戚에 孔姬使之焉한대 大子與之言曰 苟使我入獲國이면 服冕乘軒하고 三死無與하리라하고 與之盟하니 爲請于伯姬하다</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C101" t="inlineStr">
         <is>
           <t>위(衛)나라 공어(孔圉)가 태자(太子) 괴외(蒯聵)의 누이를 아내로 취하여 회(悝)를 낳았다. 공씨(孔氏)의 노복(奴僕) 혼량부(渾良夫)가 키가 크고 얼굴이 아름다웠는데, 공문자(孔文子)가 죽은 뒤에 혼량부(渾良夫)가 공문자(孔文子)의 아내 공희(孔姬)와 간통(姦通)하였다. 태자(太子)가 척(戚)에 있을 때 공희(孔姬)가 혼량부(渾良夫)를 태자(太子)에게 보내니, 태자(太子)가 혼량부(渾良夫)에게 말하기를 “만약 나로 하여금 국내(國內)로 들어가서 나라를 얻게 한다면 너를 대부(大夫)로 삼아 면관(冕冠)을 쓰고 대부(大夫)의 수레를 타게 할 것이고, 사죄(死罪)를 짓더라도 세 번은 용서할 것이다. ”라고 하고서 그와 맹약(盟約)을 맺으니, 혼량부(渾良夫)는 태자(太子)를 위하여 백희(伯姬)(공희(孔姬))에게 요청하였다.</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D101" t="inlineStr">
         <is>
           <t>춘추좌씨전8</t>
         </is>

</xml_diff>